<commit_message>
Exportação de ficha de cadastro v5
</commit_message>
<xml_diff>
--- a/backend/assets/template_supra.xlsx
+++ b/backend/assets/template_supra.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Dispet\88_Cadastros_Supra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projeto Sistema pedidos\Planejamento\Arquivos bases edson\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEBF351-9DB8-4E8E-BF7A-BC77C314219D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAEC6108-A469-4EE7-A5AC-A7F4E92CE825}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cadastro Parte 1" sheetId="5" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="116">
   <si>
     <t>COMERCIAL</t>
   </si>
@@ -324,27 +324,12 @@
     <t>USO INTERNO</t>
   </si>
   <si>
-    <t>NÃO</t>
-  </si>
-  <si>
-    <t>FILIAL 40</t>
-  </si>
-  <si>
-    <t>DISPET REPRESENTAÇÕES COMERCIAIS - CÓDIGO 178799</t>
-  </si>
-  <si>
     <t xml:space="preserve">Forma de Pagamento : </t>
   </si>
   <si>
     <t>(  ) Vendor</t>
   </si>
   <si>
-    <t>Guilherme Poerner Neto</t>
-  </si>
-  <si>
-    <t>Estado:  SP</t>
-  </si>
-  <si>
     <t>Venda a Prazo</t>
   </si>
   <si>
@@ -354,21 +339,12 @@
     <t xml:space="preserve">    Lojista = (Produto para Comercializar / Revender)</t>
   </si>
   <si>
-    <t>MATHIAS OLIVEIRA</t>
-  </si>
-  <si>
     <t xml:space="preserve">      (XX)Cobrança      </t>
   </si>
   <si>
     <t xml:space="preserve">CPF:    </t>
   </si>
   <si>
-    <t xml:space="preserve">  (X) Não</t>
-  </si>
-  <si>
-    <t>WALESKA GARCIA GAGLIANO</t>
-  </si>
-  <si>
     <t xml:space="preserve">Telefone:  </t>
   </si>
   <si>
@@ -390,106 +366,55 @@
     <t>CLIENTE NOVO</t>
   </si>
   <si>
-    <t>Nome do Cliente:  HEINRICH DEWALD PARASCHIN</t>
-  </si>
-  <si>
-    <t>Denominação Comercial/Fantasia:   ANGOLANA</t>
-  </si>
-  <si>
-    <t>Celular:  11-94233-2001</t>
-  </si>
-  <si>
     <t xml:space="preserve">E-mail:  </t>
   </si>
   <si>
-    <t>CNPJ:  22.644.122/0001-53</t>
-  </si>
-  <si>
-    <t>INSCR.  ESTADUAL:  653.080.096.119</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cli Direto:      </t>
   </si>
   <si>
-    <t>Lojista:  (XX)</t>
-  </si>
-  <si>
-    <t>Av./Rua/Nro:  ESTRADA TURISTICA ANGOLANA, Nº 1167 LOJA</t>
-  </si>
-  <si>
-    <t>CEP:  18.130-970</t>
-  </si>
-  <si>
-    <t>Bairro:  SETUBAL</t>
-  </si>
-  <si>
-    <t>Cidade:  SÃO ROQUE</t>
-  </si>
-  <si>
-    <t>C/Vendas:  HEINRICH DEWALD PARASCHIN</t>
-  </si>
-  <si>
-    <t>Telefones:  11-94233-2001</t>
-  </si>
-  <si>
-    <t>P/Cobranças:  IDEM</t>
-  </si>
-  <si>
-    <t>Telefones:  IDEM</t>
-  </si>
-  <si>
-    <t>AGROBIGA</t>
-  </si>
-  <si>
-    <t>MAIRINQUE - SP</t>
-  </si>
-  <si>
-    <t>11-4718-4343</t>
-  </si>
-  <si>
-    <t>JOAO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAKAR PNEUS </t>
-  </si>
-  <si>
-    <t>11-4712-4844</t>
-  </si>
-  <si>
-    <t>DISTRIBUIDORA MANANCIAL MAIRINQUE</t>
-  </si>
-  <si>
-    <t>11-99737-6549</t>
-  </si>
-  <si>
-    <t>MARCIO</t>
-  </si>
-  <si>
-    <t>SITIO / FAZENDINHA ANGOLANA</t>
-  </si>
-  <si>
-    <t>SÃO ROQUE - SP</t>
-  </si>
-  <si>
-    <t>3000 M A/C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRATOR </t>
-  </si>
-  <si>
-    <t>MF</t>
-  </si>
-  <si>
-    <t>SÃO ROQUE/SP, 25/3/2026</t>
-  </si>
-  <si>
-    <t>HEINRICH DEWALD PARASCHIN</t>
-  </si>
-  <si>
-    <t>ANGOLANA</t>
-  </si>
-  <si>
     <t>Utilização do Produto:   (   )Insumos na Pecuária   (   )Consumo Próprio   (   )Industrialização   (XX)Comercializar/Revender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome do Cliente:  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denominação Comercial/Fantasia:   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celular:  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CNPJ:  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">INSCR.  ESTADUAL:  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lojista: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CEP: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado:  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade:  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">C/Vendas:  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/Cobranças:  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telefones:  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telefones: </t>
+  </si>
+  <si>
+    <t>Lojista = (Produto para Comercializar / Revender)</t>
   </si>
 </sst>
 </file>
@@ -1416,6 +1341,351 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1452,363 +1722,168 @@
     <xf numFmtId="164" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1821,12 +1896,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1854,29 +1923,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1886,129 +1934,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2398,9 +2323,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2438,9 +2363,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2473,9 +2398,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2508,9 +2450,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2710,27 +2669,27 @@
     </row>
     <row r="2" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="32"/>
-      <c r="D2" s="155" t="s">
+      <c r="D2" s="67" t="s">
         <v>80</v>
       </c>
-      <c r="E2" s="155"/>
-      <c r="F2" s="155"/>
-      <c r="G2" s="155"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="155"/>
-      <c r="J2" s="155"/>
-      <c r="K2" s="156"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="32"/>
-      <c r="D3" s="155"/>
-      <c r="E3" s="155"/>
-      <c r="F3" s="155"/>
-      <c r="G3" s="155"/>
-      <c r="H3" s="155"/>
-      <c r="I3" s="155"/>
-      <c r="J3" s="155"/>
-      <c r="K3" s="156"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="68"/>
     </row>
     <row r="4" spans="1:22" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
@@ -2752,231 +2711,231 @@
       <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:22" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="167" t="s">
+      <c r="A6" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="168"/>
-      <c r="C6" s="168"/>
-      <c r="D6" s="168"/>
-      <c r="E6" s="168"/>
-      <c r="F6" s="168"/>
-      <c r="G6" s="168"/>
-      <c r="H6" s="168"/>
-      <c r="I6" s="167" t="s">
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
+      <c r="D6" s="80"/>
+      <c r="E6" s="80"/>
+      <c r="F6" s="80"/>
+      <c r="G6" s="80"/>
+      <c r="H6" s="80"/>
+      <c r="I6" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="J6" s="168"/>
-      <c r="K6" s="169"/>
+      <c r="J6" s="80"/>
+      <c r="K6" s="81"/>
     </row>
     <row r="7" spans="1:22" s="7" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="173" t="s">
+      <c r="A7" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="174"/>
-      <c r="C7" s="174"/>
-      <c r="D7" s="174"/>
-      <c r="E7" s="174"/>
-      <c r="F7" s="174"/>
-      <c r="G7" s="174"/>
-      <c r="H7" s="175"/>
-      <c r="I7" s="170" t="s">
+      <c r="B7" s="86"/>
+      <c r="C7" s="86"/>
+      <c r="D7" s="86"/>
+      <c r="E7" s="86"/>
+      <c r="F7" s="86"/>
+      <c r="G7" s="86"/>
+      <c r="H7" s="87"/>
+      <c r="I7" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="171"/>
-      <c r="K7" s="172"/>
+      <c r="J7" s="83"/>
+      <c r="K7" s="84"/>
     </row>
     <row r="8" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="176" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="177"/>
-      <c r="C8" s="177"/>
-      <c r="D8" s="177"/>
-      <c r="E8" s="177"/>
-      <c r="F8" s="177"/>
-      <c r="G8" s="177"/>
-      <c r="H8" s="178"/>
+      <c r="A8" s="88" t="s">
+        <v>102</v>
+      </c>
+      <c r="B8" s="89"/>
+      <c r="C8" s="89"/>
+      <c r="D8" s="89"/>
+      <c r="E8" s="89"/>
+      <c r="F8" s="89"/>
+      <c r="G8" s="89"/>
+      <c r="H8" s="90"/>
       <c r="I8" s="8"/>
       <c r="J8" s="9"/>
       <c r="K8" s="10"/>
-      <c r="M8" s="146" t="str">
+      <c r="M8" s="58" t="str">
         <f>'Cadastro Parte 2'!A41</f>
         <v>CLIENTE NOVO</v>
       </c>
-      <c r="N8" s="147"/>
-      <c r="O8" s="147"/>
-      <c r="P8" s="147"/>
-      <c r="Q8" s="147"/>
-      <c r="R8" s="147"/>
-      <c r="S8" s="147"/>
-      <c r="T8" s="147"/>
-      <c r="U8" s="147"/>
-      <c r="V8" s="148"/>
+      <c r="N8" s="59"/>
+      <c r="O8" s="59"/>
+      <c r="P8" s="59"/>
+      <c r="Q8" s="59"/>
+      <c r="R8" s="59"/>
+      <c r="S8" s="59"/>
+      <c r="T8" s="59"/>
+      <c r="U8" s="59"/>
+      <c r="V8" s="60"/>
     </row>
     <row r="9" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="179" t="s">
-        <v>108</v>
-      </c>
-      <c r="B9" s="180"/>
-      <c r="C9" s="180"/>
-      <c r="D9" s="180"/>
-      <c r="E9" s="180"/>
-      <c r="F9" s="180"/>
-      <c r="G9" s="180"/>
-      <c r="H9" s="181"/>
+      <c r="A9" s="91" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="92"/>
+      <c r="C9" s="92"/>
+      <c r="D9" s="92"/>
+      <c r="E9" s="92"/>
+      <c r="F9" s="92"/>
+      <c r="G9" s="92"/>
+      <c r="H9" s="93"/>
       <c r="I9" s="8" t="s">
         <v>4</v>
       </c>
       <c r="J9" s="9"/>
       <c r="K9" s="10"/>
-      <c r="M9" s="149" t="str">
+      <c r="M9" s="61" t="str">
         <f>'Cadastro Parte 2'!A42</f>
-        <v xml:space="preserve">    Lojista = (Produto para Comercializar / Revender)</v>
-      </c>
-      <c r="N9" s="150"/>
-      <c r="O9" s="150"/>
-      <c r="P9" s="150"/>
-      <c r="Q9" s="150"/>
-      <c r="R9" s="150"/>
-      <c r="S9" s="150"/>
-      <c r="T9" s="150"/>
-      <c r="U9" s="150"/>
-      <c r="V9" s="151"/>
+        <v>Lojista = (Produto para Comercializar / Revender)</v>
+      </c>
+      <c r="N9" s="62"/>
+      <c r="O9" s="62"/>
+      <c r="P9" s="62"/>
+      <c r="Q9" s="62"/>
+      <c r="R9" s="62"/>
+      <c r="S9" s="62"/>
+      <c r="T9" s="62"/>
+      <c r="U9" s="62"/>
+      <c r="V9" s="63"/>
     </row>
     <row r="10" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="179" t="s">
-        <v>100</v>
-      </c>
-      <c r="B10" s="180"/>
-      <c r="C10" s="180"/>
-      <c r="D10" s="180"/>
-      <c r="E10" s="180"/>
-      <c r="F10" s="180"/>
-      <c r="G10" s="180"/>
-      <c r="H10" s="181"/>
+      <c r="A10" s="91" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="92"/>
+      <c r="C10" s="92"/>
+      <c r="D10" s="92"/>
+      <c r="E10" s="92"/>
+      <c r="F10" s="92"/>
+      <c r="G10" s="92"/>
+      <c r="H10" s="93"/>
       <c r="I10" s="11"/>
       <c r="J10" s="12"/>
       <c r="K10" s="13"/>
-      <c r="M10" s="149" t="str">
+      <c r="M10" s="61" t="str">
         <f>'Cadastro Parte 2'!A43</f>
         <v>Venda a Prazo</v>
       </c>
-      <c r="N10" s="150"/>
-      <c r="O10" s="150"/>
-      <c r="P10" s="150"/>
-      <c r="Q10" s="150"/>
-      <c r="R10" s="150"/>
-      <c r="S10" s="150"/>
-      <c r="T10" s="150"/>
-      <c r="U10" s="150"/>
-      <c r="V10" s="151"/>
+      <c r="N10" s="62"/>
+      <c r="O10" s="62"/>
+      <c r="P10" s="62"/>
+      <c r="Q10" s="62"/>
+      <c r="R10" s="62"/>
+      <c r="S10" s="62"/>
+      <c r="T10" s="62"/>
+      <c r="U10" s="62"/>
+      <c r="V10" s="63"/>
     </row>
     <row r="11" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="182" t="s">
-        <v>109</v>
-      </c>
-      <c r="B11" s="183"/>
-      <c r="C11" s="183"/>
-      <c r="D11" s="183"/>
-      <c r="E11" s="157" t="s">
-        <v>110</v>
-      </c>
-      <c r="F11" s="158"/>
-      <c r="G11" s="158"/>
-      <c r="H11" s="158"/>
-      <c r="I11" s="158"/>
-      <c r="J11" s="158"/>
-      <c r="K11" s="159"/>
-      <c r="M11" s="149">
+      <c r="A11" s="94" t="s">
+        <v>104</v>
+      </c>
+      <c r="B11" s="95"/>
+      <c r="C11" s="95"/>
+      <c r="D11" s="95"/>
+      <c r="E11" s="69" t="s">
+        <v>99</v>
+      </c>
+      <c r="F11" s="70"/>
+      <c r="G11" s="70"/>
+      <c r="H11" s="70"/>
+      <c r="I11" s="70"/>
+      <c r="J11" s="70"/>
+      <c r="K11" s="71"/>
+      <c r="M11" s="61">
         <f>'Cadastro Parte 2'!A44</f>
         <v>0</v>
       </c>
-      <c r="N11" s="150"/>
-      <c r="O11" s="150"/>
-      <c r="P11" s="150"/>
-      <c r="Q11" s="150"/>
-      <c r="R11" s="150"/>
-      <c r="S11" s="150"/>
-      <c r="T11" s="150"/>
-      <c r="U11" s="150"/>
-      <c r="V11" s="151"/>
+      <c r="N11" s="62"/>
+      <c r="O11" s="62"/>
+      <c r="P11" s="62"/>
+      <c r="Q11" s="62"/>
+      <c r="R11" s="62"/>
+      <c r="S11" s="62"/>
+      <c r="T11" s="62"/>
+      <c r="U11" s="62"/>
+      <c r="V11" s="63"/>
     </row>
     <row r="12" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="182" t="s">
-        <v>111</v>
-      </c>
-      <c r="B12" s="183"/>
-      <c r="C12" s="183"/>
-      <c r="D12" s="183"/>
-      <c r="E12" s="184" t="s">
+      <c r="A12" s="94" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="96" t="s">
         <v>67</v>
       </c>
-      <c r="F12" s="184"/>
-      <c r="G12" s="184"/>
-      <c r="H12" s="184"/>
-      <c r="I12" s="184"/>
-      <c r="J12" s="184"/>
-      <c r="K12" s="185"/>
-      <c r="M12" s="152">
+      <c r="F12" s="96"/>
+      <c r="G12" s="96"/>
+      <c r="H12" s="96"/>
+      <c r="I12" s="96"/>
+      <c r="J12" s="96"/>
+      <c r="K12" s="97"/>
+      <c r="M12" s="64">
         <f>'Cadastro Parte 2'!A45</f>
         <v>0</v>
       </c>
-      <c r="N12" s="153"/>
-      <c r="O12" s="153"/>
-      <c r="P12" s="153"/>
-      <c r="Q12" s="153"/>
-      <c r="R12" s="153"/>
-      <c r="S12" s="153"/>
-      <c r="T12" s="153"/>
-      <c r="U12" s="153"/>
-      <c r="V12" s="154"/>
+      <c r="N12" s="65"/>
+      <c r="O12" s="65"/>
+      <c r="P12" s="65"/>
+      <c r="Q12" s="65"/>
+      <c r="R12" s="65"/>
+      <c r="S12" s="65"/>
+      <c r="T12" s="65"/>
+      <c r="U12" s="65"/>
+      <c r="V12" s="66"/>
     </row>
     <row r="13" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="182" t="s">
-        <v>97</v>
-      </c>
-      <c r="B13" s="183"/>
-      <c r="C13" s="183"/>
-      <c r="D13" s="183"/>
-      <c r="E13" s="183" t="s">
-        <v>112</v>
-      </c>
-      <c r="F13" s="183"/>
-      <c r="G13" s="183"/>
-      <c r="H13" s="183"/>
-      <c r="I13" s="183"/>
-      <c r="J13" s="183"/>
-      <c r="K13" s="186"/>
+      <c r="A13" s="94" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="95"/>
+      <c r="C13" s="95"/>
+      <c r="D13" s="95"/>
+      <c r="E13" s="95" t="s">
+        <v>106</v>
+      </c>
+      <c r="F13" s="95"/>
+      <c r="G13" s="95"/>
+      <c r="H13" s="95"/>
+      <c r="I13" s="95"/>
+      <c r="J13" s="95"/>
+      <c r="K13" s="98"/>
     </row>
     <row r="14" spans="1:22" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="136" t="s">
+      <c r="A14" s="103" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="137"/>
-      <c r="C14" s="137"/>
-      <c r="D14" s="137"/>
-      <c r="E14" s="137"/>
-      <c r="F14" s="137"/>
-      <c r="G14" s="137"/>
-      <c r="H14" s="137"/>
-      <c r="I14" s="137"/>
-      <c r="J14" s="137"/>
-      <c r="K14" s="138"/>
+      <c r="B14" s="104"/>
+      <c r="C14" s="104"/>
+      <c r="D14" s="104"/>
+      <c r="E14" s="104"/>
+      <c r="F14" s="104"/>
+      <c r="G14" s="104"/>
+      <c r="H14" s="104"/>
+      <c r="I14" s="104"/>
+      <c r="J14" s="104"/>
+      <c r="K14" s="105"/>
     </row>
     <row r="15" spans="1:22" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="160" t="s">
+      <c r="A15" s="72" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="161"/>
-      <c r="C15" s="161"/>
-      <c r="D15" s="161"/>
-      <c r="E15" s="161"/>
-      <c r="F15" s="161"/>
-      <c r="G15" s="161"/>
-      <c r="H15" s="161"/>
-      <c r="I15" s="161"/>
-      <c r="J15" s="161"/>
-      <c r="K15" s="162"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
+      <c r="H15" s="73"/>
+      <c r="I15" s="73"/>
+      <c r="J15" s="73"/>
+      <c r="K15" s="74"/>
     </row>
     <row r="16" spans="1:22" s="7" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="35" t="s">
@@ -2994,48 +2953,48 @@
       <c r="K16" s="28"/>
     </row>
     <row r="17" spans="1:11" s="7" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="132" t="s">
+      <c r="A17" s="99" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="133"/>
-      <c r="C17" s="163" t="s">
+      <c r="B17" s="100"/>
+      <c r="C17" s="75" t="s">
         <v>70</v>
       </c>
-      <c r="D17" s="164"/>
-      <c r="E17" s="163" t="s">
-        <v>113</v>
-      </c>
-      <c r="F17" s="164"/>
-      <c r="G17" s="163" t="s">
+      <c r="D17" s="76"/>
+      <c r="E17" s="75" t="s">
+        <v>100</v>
+      </c>
+      <c r="F17" s="76"/>
+      <c r="G17" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="H17" s="164"/>
-      <c r="I17" s="163" t="s">
+      <c r="H17" s="76"/>
+      <c r="I17" s="75" t="s">
         <v>74</v>
       </c>
-      <c r="J17" s="165"/>
-      <c r="K17" s="166"/>
+      <c r="J17" s="77"/>
+      <c r="K17" s="78"/>
     </row>
     <row r="18" spans="1:11" s="7" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="134"/>
-      <c r="B18" s="135"/>
-      <c r="C18" s="139" t="s">
-        <v>114</v>
-      </c>
-      <c r="D18" s="140"/>
-      <c r="E18" s="139" t="s">
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="106" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18" s="107"/>
+      <c r="E18" s="106" t="s">
         <v>71</v>
       </c>
-      <c r="F18" s="140"/>
-      <c r="G18" s="139" t="s">
+      <c r="F18" s="107"/>
+      <c r="G18" s="106" t="s">
         <v>73</v>
       </c>
-      <c r="H18" s="140"/>
-      <c r="I18" s="139" t="s">
+      <c r="H18" s="107"/>
+      <c r="I18" s="106" t="s">
         <v>75</v>
       </c>
-      <c r="J18" s="141"/>
-      <c r="K18" s="142"/>
+      <c r="J18" s="117"/>
+      <c r="K18" s="118"/>
     </row>
     <row r="19" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="50"/>
@@ -3051,55 +3010,55 @@
       <c r="K19" s="46"/>
     </row>
     <row r="20" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="93" t="s">
+      <c r="A20" s="111" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="94"/>
-      <c r="C20" s="94"/>
-      <c r="D20" s="94"/>
-      <c r="E20" s="94"/>
-      <c r="F20" s="94"/>
-      <c r="G20" s="94"/>
-      <c r="H20" s="94"/>
-      <c r="I20" s="94"/>
-      <c r="J20" s="94"/>
-      <c r="K20" s="95"/>
+      <c r="B20" s="112"/>
+      <c r="C20" s="112"/>
+      <c r="D20" s="112"/>
+      <c r="E20" s="112"/>
+      <c r="F20" s="112"/>
+      <c r="G20" s="112"/>
+      <c r="H20" s="112"/>
+      <c r="I20" s="112"/>
+      <c r="J20" s="112"/>
+      <c r="K20" s="113"/>
     </row>
     <row r="21" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="143" t="s">
-        <v>115</v>
-      </c>
-      <c r="B21" s="144"/>
-      <c r="C21" s="144"/>
-      <c r="D21" s="144"/>
-      <c r="E21" s="144"/>
-      <c r="F21" s="144"/>
-      <c r="G21" s="144"/>
-      <c r="H21" s="145"/>
-      <c r="I21" s="119" t="s">
-        <v>116</v>
-      </c>
-      <c r="J21" s="120"/>
-      <c r="K21" s="121"/>
+      <c r="A21" s="119" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" s="120"/>
+      <c r="C21" s="120"/>
+      <c r="D21" s="120"/>
+      <c r="E21" s="120"/>
+      <c r="F21" s="120"/>
+      <c r="G21" s="120"/>
+      <c r="H21" s="121"/>
+      <c r="I21" s="122" t="s">
+        <v>108</v>
+      </c>
+      <c r="J21" s="123"/>
+      <c r="K21" s="124"/>
     </row>
     <row r="22" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="83" t="s">
-        <v>117</v>
-      </c>
-      <c r="B22" s="84"/>
-      <c r="C22" s="84"/>
-      <c r="D22" s="84"/>
-      <c r="E22" s="84"/>
-      <c r="F22" s="122" t="s">
-        <v>118</v>
-      </c>
-      <c r="G22" s="84"/>
-      <c r="H22" s="85"/>
-      <c r="I22" s="122" t="s">
-        <v>91</v>
-      </c>
-      <c r="J22" s="84"/>
-      <c r="K22" s="123"/>
+      <c r="A22" s="108" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" s="109"/>
+      <c r="C22" s="109"/>
+      <c r="D22" s="109"/>
+      <c r="E22" s="109"/>
+      <c r="F22" s="114" t="s">
+        <v>110</v>
+      </c>
+      <c r="G22" s="109"/>
+      <c r="H22" s="115"/>
+      <c r="I22" s="114" t="s">
+        <v>109</v>
+      </c>
+      <c r="J22" s="109"/>
+      <c r="K22" s="116"/>
     </row>
     <row r="23" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="50"/>
@@ -3115,55 +3074,55 @@
       <c r="K23" s="48"/>
     </row>
     <row r="24" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="93" t="s">
+      <c r="A24" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="94"/>
-      <c r="C24" s="94"/>
-      <c r="D24" s="94"/>
-      <c r="E24" s="94"/>
-      <c r="F24" s="94"/>
-      <c r="G24" s="94"/>
-      <c r="H24" s="94"/>
-      <c r="I24" s="94"/>
-      <c r="J24" s="94"/>
-      <c r="K24" s="95"/>
+      <c r="B24" s="112"/>
+      <c r="C24" s="112"/>
+      <c r="D24" s="112"/>
+      <c r="E24" s="112"/>
+      <c r="F24" s="112"/>
+      <c r="G24" s="112"/>
+      <c r="H24" s="112"/>
+      <c r="I24" s="112"/>
+      <c r="J24" s="112"/>
+      <c r="K24" s="113"/>
     </row>
     <row r="25" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="126" t="s">
-        <v>101</v>
-      </c>
-      <c r="B25" s="127"/>
-      <c r="C25" s="127"/>
-      <c r="D25" s="127"/>
-      <c r="E25" s="127"/>
-      <c r="F25" s="127"/>
-      <c r="G25" s="127"/>
-      <c r="H25" s="128"/>
-      <c r="I25" s="119" t="s">
-        <v>102</v>
-      </c>
-      <c r="J25" s="120"/>
-      <c r="K25" s="121"/>
+      <c r="A25" s="132" t="s">
+        <v>93</v>
+      </c>
+      <c r="B25" s="133"/>
+      <c r="C25" s="133"/>
+      <c r="D25" s="133"/>
+      <c r="E25" s="133"/>
+      <c r="F25" s="133"/>
+      <c r="G25" s="133"/>
+      <c r="H25" s="134"/>
+      <c r="I25" s="122" t="s">
+        <v>94</v>
+      </c>
+      <c r="J25" s="123"/>
+      <c r="K25" s="124"/>
     </row>
     <row r="26" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="83" t="s">
-        <v>103</v>
-      </c>
-      <c r="B26" s="84"/>
-      <c r="C26" s="84"/>
-      <c r="D26" s="84"/>
-      <c r="E26" s="84"/>
-      <c r="F26" s="122" t="s">
-        <v>104</v>
-      </c>
-      <c r="G26" s="84"/>
-      <c r="H26" s="85"/>
-      <c r="I26" s="122" t="s">
-        <v>105</v>
-      </c>
-      <c r="J26" s="84"/>
-      <c r="K26" s="123"/>
+      <c r="A26" s="108" t="s">
+        <v>95</v>
+      </c>
+      <c r="B26" s="109"/>
+      <c r="C26" s="109"/>
+      <c r="D26" s="109"/>
+      <c r="E26" s="109"/>
+      <c r="F26" s="114" t="s">
+        <v>96</v>
+      </c>
+      <c r="G26" s="109"/>
+      <c r="H26" s="115"/>
+      <c r="I26" s="114" t="s">
+        <v>97</v>
+      </c>
+      <c r="J26" s="109"/>
+      <c r="K26" s="116"/>
     </row>
     <row r="27" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="50"/>
@@ -3179,53 +3138,53 @@
       <c r="K27" s="48"/>
     </row>
     <row r="28" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="93" t="s">
+      <c r="A28" s="111" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="94"/>
-      <c r="F28" s="94"/>
-      <c r="G28" s="94"/>
-      <c r="H28" s="94"/>
-      <c r="I28" s="94"/>
-      <c r="J28" s="94"/>
-      <c r="K28" s="95"/>
+      <c r="B28" s="112"/>
+      <c r="C28" s="112"/>
+      <c r="D28" s="112"/>
+      <c r="E28" s="112"/>
+      <c r="F28" s="112"/>
+      <c r="G28" s="112"/>
+      <c r="H28" s="112"/>
+      <c r="I28" s="112"/>
+      <c r="J28" s="112"/>
+      <c r="K28" s="113"/>
     </row>
     <row r="29" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="124" t="s">
-        <v>119</v>
-      </c>
-      <c r="B29" s="125"/>
-      <c r="C29" s="125"/>
-      <c r="D29" s="125"/>
-      <c r="E29" s="125"/>
-      <c r="F29" s="119" t="s">
-        <v>120</v>
-      </c>
-      <c r="G29" s="120"/>
-      <c r="H29" s="120"/>
-      <c r="I29" s="120"/>
-      <c r="J29" s="120"/>
-      <c r="K29" s="121"/>
+      <c r="A29" s="130" t="s">
+        <v>111</v>
+      </c>
+      <c r="B29" s="131"/>
+      <c r="C29" s="131"/>
+      <c r="D29" s="131"/>
+      <c r="E29" s="131"/>
+      <c r="F29" s="122" t="s">
+        <v>113</v>
+      </c>
+      <c r="G29" s="123"/>
+      <c r="H29" s="123"/>
+      <c r="I29" s="123"/>
+      <c r="J29" s="123"/>
+      <c r="K29" s="124"/>
     </row>
     <row r="30" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="72" t="s">
-        <v>121</v>
-      </c>
-      <c r="B30" s="73"/>
-      <c r="C30" s="73"/>
-      <c r="D30" s="73"/>
-      <c r="E30" s="73"/>
-      <c r="F30" s="129" t="s">
-        <v>122</v>
-      </c>
-      <c r="G30" s="130"/>
-      <c r="H30" s="130"/>
-      <c r="I30" s="130"/>
-      <c r="J30" s="130"/>
-      <c r="K30" s="131"/>
+      <c r="A30" s="139" t="s">
+        <v>112</v>
+      </c>
+      <c r="B30" s="140"/>
+      <c r="C30" s="140"/>
+      <c r="D30" s="140"/>
+      <c r="E30" s="140"/>
+      <c r="F30" s="141" t="s">
+        <v>114</v>
+      </c>
+      <c r="G30" s="142"/>
+      <c r="H30" s="142"/>
+      <c r="I30" s="142"/>
+      <c r="J30" s="142"/>
+      <c r="K30" s="143"/>
     </row>
     <row r="31" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="50"/>
@@ -3241,83 +3200,83 @@
       <c r="K31" s="48"/>
     </row>
     <row r="32" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="93" t="s">
+      <c r="A32" s="111" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="94"/>
-      <c r="C32" s="94"/>
-      <c r="D32" s="94"/>
-      <c r="E32" s="94"/>
-      <c r="F32" s="94"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="94"/>
-      <c r="I32" s="94"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="95"/>
+      <c r="B32" s="112"/>
+      <c r="C32" s="112"/>
+      <c r="D32" s="112"/>
+      <c r="E32" s="112"/>
+      <c r="F32" s="112"/>
+      <c r="G32" s="112"/>
+      <c r="H32" s="112"/>
+      <c r="I32" s="112"/>
+      <c r="J32" s="112"/>
+      <c r="K32" s="113"/>
     </row>
     <row r="33" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="117" t="s">
+      <c r="A33" s="128" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="118"/>
-      <c r="C33" s="97" t="s">
+      <c r="B33" s="129"/>
+      <c r="C33" s="110" t="s">
         <v>12</v>
       </c>
-      <c r="D33" s="97"/>
-      <c r="E33" s="97" t="s">
+      <c r="D33" s="110"/>
+      <c r="E33" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="F33" s="97"/>
+      <c r="F33" s="110"/>
       <c r="G33" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="H33" s="97" t="s">
+      <c r="H33" s="110" t="s">
         <v>14</v>
       </c>
-      <c r="I33" s="97"/>
-      <c r="J33" s="97" t="s">
+      <c r="I33" s="110"/>
+      <c r="J33" s="110" t="s">
         <v>15</v>
       </c>
-      <c r="K33" s="98"/>
+      <c r="K33" s="126"/>
     </row>
     <row r="34" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="77"/>
-      <c r="B34" s="78"/>
-      <c r="C34" s="87"/>
-      <c r="D34" s="88"/>
-      <c r="E34" s="87"/>
-      <c r="F34" s="88"/>
+      <c r="A34" s="137"/>
+      <c r="B34" s="138"/>
+      <c r="C34" s="135"/>
+      <c r="D34" s="136"/>
+      <c r="E34" s="135"/>
+      <c r="F34" s="136"/>
       <c r="G34" s="55"/>
-      <c r="H34" s="70"/>
-      <c r="I34" s="70"/>
-      <c r="J34" s="70"/>
-      <c r="K34" s="71"/>
+      <c r="H34" s="125"/>
+      <c r="I34" s="125"/>
+      <c r="J34" s="125"/>
+      <c r="K34" s="127"/>
     </row>
     <row r="35" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="77"/>
-      <c r="B35" s="78"/>
-      <c r="C35" s="70"/>
-      <c r="D35" s="70"/>
-      <c r="E35" s="70"/>
-      <c r="F35" s="70"/>
+      <c r="A35" s="137"/>
+      <c r="B35" s="138"/>
+      <c r="C35" s="125"/>
+      <c r="D35" s="125"/>
+      <c r="E35" s="125"/>
+      <c r="F35" s="125"/>
       <c r="G35" s="55"/>
-      <c r="H35" s="70"/>
-      <c r="I35" s="70"/>
-      <c r="J35" s="70"/>
-      <c r="K35" s="71"/>
+      <c r="H35" s="125"/>
+      <c r="I35" s="125"/>
+      <c r="J35" s="125"/>
+      <c r="K35" s="127"/>
     </row>
     <row r="36" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="72"/>
-      <c r="B36" s="73"/>
-      <c r="C36" s="75"/>
-      <c r="D36" s="75"/>
-      <c r="E36" s="75"/>
-      <c r="F36" s="75"/>
+      <c r="A36" s="139"/>
+      <c r="B36" s="140"/>
+      <c r="C36" s="145"/>
+      <c r="D36" s="145"/>
+      <c r="E36" s="145"/>
+      <c r="F36" s="145"/>
       <c r="G36" s="56"/>
-      <c r="H36" s="75"/>
-      <c r="I36" s="75"/>
-      <c r="J36" s="75"/>
-      <c r="K36" s="76"/>
+      <c r="H36" s="145"/>
+      <c r="I36" s="145"/>
+      <c r="J36" s="145"/>
+      <c r="K36" s="146"/>
     </row>
     <row r="37" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="50"/>
@@ -3333,101 +3292,79 @@
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="93" t="s">
+      <c r="A38" s="111" t="s">
         <v>18</v>
       </c>
-      <c r="B38" s="94"/>
-      <c r="C38" s="94"/>
-      <c r="D38" s="94"/>
-      <c r="E38" s="94"/>
-      <c r="F38" s="94"/>
-      <c r="G38" s="94"/>
-      <c r="H38" s="94"/>
-      <c r="I38" s="94"/>
-      <c r="J38" s="94"/>
-      <c r="K38" s="95"/>
+      <c r="B38" s="112"/>
+      <c r="C38" s="112"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="112"/>
+      <c r="G38" s="112"/>
+      <c r="H38" s="112"/>
+      <c r="I38" s="112"/>
+      <c r="J38" s="112"/>
+      <c r="K38" s="113"/>
     </row>
     <row r="39" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="96" t="s">
+      <c r="A39" s="144" t="s">
         <v>19</v>
       </c>
-      <c r="B39" s="97"/>
-      <c r="C39" s="97"/>
-      <c r="D39" s="97"/>
-      <c r="E39" s="97" t="s">
+      <c r="B39" s="110"/>
+      <c r="C39" s="110"/>
+      <c r="D39" s="110"/>
+      <c r="E39" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="F39" s="97"/>
-      <c r="G39" s="97" t="s">
+      <c r="F39" s="110"/>
+      <c r="G39" s="110" t="s">
         <v>14</v>
       </c>
-      <c r="H39" s="97"/>
-      <c r="I39" s="97" t="s">
+      <c r="H39" s="110"/>
+      <c r="I39" s="110" t="s">
         <v>15</v>
       </c>
-      <c r="J39" s="97"/>
-      <c r="K39" s="98"/>
+      <c r="J39" s="110"/>
+      <c r="K39" s="126"/>
     </row>
     <row r="40" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="113" t="s">
-        <v>123</v>
-      </c>
-      <c r="B40" s="114"/>
-      <c r="C40" s="114"/>
-      <c r="D40" s="115"/>
-      <c r="E40" s="87" t="s">
-        <v>124</v>
-      </c>
-      <c r="F40" s="88"/>
-      <c r="G40" s="87" t="s">
-        <v>125</v>
-      </c>
-      <c r="H40" s="88"/>
-      <c r="I40" s="87" t="s">
-        <v>126</v>
-      </c>
-      <c r="J40" s="116"/>
-      <c r="K40" s="91"/>
+      <c r="A40" s="154"/>
+      <c r="B40" s="155"/>
+      <c r="C40" s="155"/>
+      <c r="D40" s="156"/>
+      <c r="E40" s="135"/>
+      <c r="F40" s="136"/>
+      <c r="G40" s="135"/>
+      <c r="H40" s="136"/>
+      <c r="I40" s="135"/>
+      <c r="J40" s="157"/>
+      <c r="K40" s="158"/>
     </row>
     <row r="41" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="113" t="s">
-        <v>127</v>
-      </c>
-      <c r="B41" s="114"/>
-      <c r="C41" s="114"/>
-      <c r="D41" s="115"/>
-      <c r="E41" s="87" t="s">
-        <v>124</v>
-      </c>
-      <c r="F41" s="88"/>
-      <c r="G41" s="87" t="s">
-        <v>128</v>
-      </c>
-      <c r="H41" s="88"/>
-      <c r="I41" s="87"/>
-      <c r="J41" s="116"/>
-      <c r="K41" s="91"/>
+      <c r="A41" s="154"/>
+      <c r="B41" s="155"/>
+      <c r="C41" s="155"/>
+      <c r="D41" s="156"/>
+      <c r="E41" s="135"/>
+      <c r="F41" s="136"/>
+      <c r="G41" s="135"/>
+      <c r="H41" s="136"/>
+      <c r="I41" s="135"/>
+      <c r="J41" s="157"/>
+      <c r="K41" s="158"/>
     </row>
     <row r="42" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="106" t="s">
-        <v>129</v>
-      </c>
-      <c r="B42" s="107"/>
-      <c r="C42" s="107"/>
-      <c r="D42" s="108"/>
-      <c r="E42" s="109" t="s">
-        <v>124</v>
-      </c>
-      <c r="F42" s="110"/>
-      <c r="G42" s="109" t="s">
-        <v>130</v>
-      </c>
-      <c r="H42" s="110"/>
-      <c r="I42" s="109" t="s">
-        <v>131</v>
-      </c>
-      <c r="J42" s="111"/>
-      <c r="K42" s="112"/>
+      <c r="A42" s="147"/>
+      <c r="B42" s="148"/>
+      <c r="C42" s="148"/>
+      <c r="D42" s="149"/>
+      <c r="E42" s="150"/>
+      <c r="F42" s="151"/>
+      <c r="G42" s="150"/>
+      <c r="H42" s="151"/>
+      <c r="I42" s="150"/>
+      <c r="J42" s="152"/>
+      <c r="K42" s="153"/>
     </row>
     <row r="43" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="50"/>
@@ -3443,80 +3380,68 @@
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="93" t="s">
+      <c r="A44" s="111" t="s">
         <v>21</v>
       </c>
-      <c r="B44" s="94"/>
-      <c r="C44" s="94"/>
-      <c r="D44" s="94"/>
-      <c r="E44" s="94"/>
-      <c r="F44" s="94"/>
-      <c r="G44" s="94"/>
-      <c r="H44" s="94"/>
-      <c r="I44" s="94"/>
-      <c r="J44" s="94"/>
-      <c r="K44" s="95"/>
+      <c r="B44" s="112"/>
+      <c r="C44" s="112"/>
+      <c r="D44" s="112"/>
+      <c r="E44" s="112"/>
+      <c r="F44" s="112"/>
+      <c r="G44" s="112"/>
+      <c r="H44" s="112"/>
+      <c r="I44" s="112"/>
+      <c r="J44" s="112"/>
+      <c r="K44" s="113"/>
     </row>
     <row r="45" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="96" t="s">
+      <c r="A45" s="144" t="s">
         <v>22</v>
       </c>
-      <c r="B45" s="97"/>
-      <c r="C45" s="97" t="s">
+      <c r="B45" s="110"/>
+      <c r="C45" s="110" t="s">
         <v>23</v>
       </c>
-      <c r="D45" s="97"/>
-      <c r="E45" s="97"/>
-      <c r="F45" s="97" t="s">
+      <c r="D45" s="110"/>
+      <c r="E45" s="110"/>
+      <c r="F45" s="110" t="s">
         <v>24</v>
       </c>
-      <c r="G45" s="97"/>
-      <c r="H45" s="97" t="s">
+      <c r="G45" s="110"/>
+      <c r="H45" s="110" t="s">
         <v>35</v>
       </c>
-      <c r="I45" s="97"/>
-      <c r="J45" s="97" t="s">
+      <c r="I45" s="110"/>
+      <c r="J45" s="110" t="s">
         <v>26</v>
       </c>
-      <c r="K45" s="98"/>
+      <c r="K45" s="126"/>
     </row>
     <row r="46" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="80" t="s">
-        <v>132</v>
-      </c>
-      <c r="B46" s="82"/>
-      <c r="C46" s="70" t="s">
-        <v>133</v>
-      </c>
-      <c r="D46" s="70"/>
-      <c r="E46" s="70"/>
-      <c r="F46" s="70" t="s">
-        <v>134</v>
-      </c>
-      <c r="G46" s="70"/>
-      <c r="H46" s="105">
-        <v>15000000</v>
-      </c>
-      <c r="I46" s="105"/>
-      <c r="J46" s="70" t="s">
-        <v>85</v>
-      </c>
-      <c r="K46" s="71"/>
+      <c r="A46" s="160"/>
+      <c r="B46" s="161"/>
+      <c r="C46" s="125"/>
+      <c r="D46" s="125"/>
+      <c r="E46" s="125"/>
+      <c r="F46" s="125"/>
+      <c r="G46" s="125"/>
+      <c r="H46" s="162"/>
+      <c r="I46" s="162"/>
+      <c r="J46" s="125"/>
+      <c r="K46" s="127"/>
     </row>
     <row r="47" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="83"/>
-      <c r="B47" s="85"/>
-      <c r="C47" s="75"/>
-      <c r="D47" s="75"/>
-      <c r="E47" s="75"/>
-      <c r="F47" s="75"/>
-      <c r="G47" s="75"/>
-      <c r="H47" s="104"/>
-      <c r="I47" s="104"/>
-      <c r="J47" s="75" t="s">
-        <v>85</v>
-      </c>
-      <c r="K47" s="76"/>
+      <c r="A47" s="108"/>
+      <c r="B47" s="115"/>
+      <c r="C47" s="145"/>
+      <c r="D47" s="145"/>
+      <c r="E47" s="145"/>
+      <c r="F47" s="145"/>
+      <c r="G47" s="145"/>
+      <c r="H47" s="159"/>
+      <c r="I47" s="159"/>
+      <c r="J47" s="145"/>
+      <c r="K47" s="146"/>
     </row>
     <row r="48" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="50"/>
@@ -3532,79 +3457,79 @@
       <c r="K48" s="51"/>
     </row>
     <row r="49" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="93" t="s">
+      <c r="A49" s="111" t="s">
         <v>27</v>
       </c>
-      <c r="B49" s="94"/>
-      <c r="C49" s="94"/>
-      <c r="D49" s="94"/>
-      <c r="E49" s="94"/>
-      <c r="F49" s="94"/>
-      <c r="G49" s="94"/>
-      <c r="H49" s="94"/>
-      <c r="I49" s="94"/>
-      <c r="J49" s="94"/>
-      <c r="K49" s="95"/>
+      <c r="B49" s="112"/>
+      <c r="C49" s="112"/>
+      <c r="D49" s="112"/>
+      <c r="E49" s="112"/>
+      <c r="F49" s="112"/>
+      <c r="G49" s="112"/>
+      <c r="H49" s="112"/>
+      <c r="I49" s="112"/>
+      <c r="J49" s="112"/>
+      <c r="K49" s="113"/>
     </row>
     <row r="50" spans="1:11" s="7" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="99" t="s">
+      <c r="A50" s="163" t="s">
         <v>28</v>
       </c>
-      <c r="B50" s="100"/>
-      <c r="C50" s="100"/>
-      <c r="D50" s="100"/>
-      <c r="E50" s="100"/>
-      <c r="F50" s="100" t="s">
+      <c r="B50" s="164"/>
+      <c r="C50" s="164"/>
+      <c r="D50" s="164"/>
+      <c r="E50" s="164"/>
+      <c r="F50" s="164" t="s">
         <v>29</v>
       </c>
-      <c r="G50" s="100"/>
-      <c r="H50" s="101" t="s">
+      <c r="G50" s="164"/>
+      <c r="H50" s="166" t="s">
         <v>76</v>
       </c>
-      <c r="I50" s="102"/>
-      <c r="J50" s="101" t="s">
+      <c r="I50" s="167"/>
+      <c r="J50" s="166" t="s">
         <v>77</v>
       </c>
-      <c r="K50" s="103"/>
+      <c r="K50" s="168"/>
     </row>
     <row r="51" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="80"/>
-      <c r="B51" s="81"/>
-      <c r="C51" s="81"/>
-      <c r="D51" s="81"/>
-      <c r="E51" s="82"/>
-      <c r="F51" s="70"/>
-      <c r="G51" s="70"/>
-      <c r="H51" s="87"/>
-      <c r="I51" s="88"/>
-      <c r="J51" s="87"/>
-      <c r="K51" s="91"/>
+      <c r="A51" s="160"/>
+      <c r="B51" s="165"/>
+      <c r="C51" s="165"/>
+      <c r="D51" s="165"/>
+      <c r="E51" s="161"/>
+      <c r="F51" s="125"/>
+      <c r="G51" s="125"/>
+      <c r="H51" s="135"/>
+      <c r="I51" s="136"/>
+      <c r="J51" s="135"/>
+      <c r="K51" s="158"/>
     </row>
     <row r="52" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="80"/>
-      <c r="B52" s="81"/>
-      <c r="C52" s="81"/>
-      <c r="D52" s="81"/>
-      <c r="E52" s="82"/>
-      <c r="F52" s="70"/>
-      <c r="G52" s="70"/>
-      <c r="H52" s="87"/>
-      <c r="I52" s="88"/>
-      <c r="J52" s="87"/>
-      <c r="K52" s="91"/>
+      <c r="A52" s="160"/>
+      <c r="B52" s="165"/>
+      <c r="C52" s="165"/>
+      <c r="D52" s="165"/>
+      <c r="E52" s="161"/>
+      <c r="F52" s="125"/>
+      <c r="G52" s="125"/>
+      <c r="H52" s="135"/>
+      <c r="I52" s="136"/>
+      <c r="J52" s="135"/>
+      <c r="K52" s="158"/>
     </row>
     <row r="53" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="83"/>
-      <c r="B53" s="84"/>
-      <c r="C53" s="84"/>
-      <c r="D53" s="84"/>
-      <c r="E53" s="85"/>
-      <c r="F53" s="75"/>
-      <c r="G53" s="75"/>
-      <c r="H53" s="89"/>
-      <c r="I53" s="90"/>
-      <c r="J53" s="89"/>
-      <c r="K53" s="92"/>
+      <c r="A53" s="108"/>
+      <c r="B53" s="109"/>
+      <c r="C53" s="109"/>
+      <c r="D53" s="109"/>
+      <c r="E53" s="115"/>
+      <c r="F53" s="145"/>
+      <c r="G53" s="145"/>
+      <c r="H53" s="170"/>
+      <c r="I53" s="171"/>
+      <c r="J53" s="170"/>
+      <c r="K53" s="172"/>
     </row>
     <row r="54" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="52"/>
@@ -3620,119 +3545,109 @@
       <c r="K54" s="51"/>
     </row>
     <row r="55" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="93" t="s">
+      <c r="A55" s="111" t="s">
         <v>53</v>
       </c>
-      <c r="B55" s="94"/>
-      <c r="C55" s="94"/>
-      <c r="D55" s="94"/>
-      <c r="E55" s="94"/>
-      <c r="F55" s="94"/>
-      <c r="G55" s="94"/>
-      <c r="H55" s="94"/>
-      <c r="I55" s="94"/>
-      <c r="J55" s="94"/>
-      <c r="K55" s="95"/>
+      <c r="B55" s="112"/>
+      <c r="C55" s="112"/>
+      <c r="D55" s="112"/>
+      <c r="E55" s="112"/>
+      <c r="F55" s="112"/>
+      <c r="G55" s="112"/>
+      <c r="H55" s="112"/>
+      <c r="I55" s="112"/>
+      <c r="J55" s="112"/>
+      <c r="K55" s="113"/>
     </row>
     <row r="56" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="96" t="s">
+      <c r="A56" s="144" t="s">
         <v>30</v>
       </c>
-      <c r="B56" s="97"/>
-      <c r="C56" s="97"/>
-      <c r="D56" s="97"/>
-      <c r="E56" s="97" t="s">
+      <c r="B56" s="110"/>
+      <c r="C56" s="110"/>
+      <c r="D56" s="110"/>
+      <c r="E56" s="110" t="s">
         <v>31</v>
       </c>
-      <c r="F56" s="97"/>
-      <c r="G56" s="97" t="s">
+      <c r="F56" s="110"/>
+      <c r="G56" s="110" t="s">
         <v>25</v>
       </c>
-      <c r="H56" s="97"/>
-      <c r="I56" s="97" t="s">
+      <c r="H56" s="110"/>
+      <c r="I56" s="110" t="s">
         <v>32</v>
       </c>
-      <c r="J56" s="97"/>
-      <c r="K56" s="98"/>
+      <c r="J56" s="110"/>
+      <c r="K56" s="126"/>
     </row>
     <row r="57" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="77" t="s">
-        <v>135</v>
-      </c>
-      <c r="B57" s="78"/>
-      <c r="C57" s="78"/>
-      <c r="D57" s="78"/>
-      <c r="E57" s="70" t="s">
-        <v>136</v>
-      </c>
-      <c r="F57" s="70"/>
-      <c r="G57" s="86">
-        <v>0</v>
-      </c>
-      <c r="H57" s="86"/>
-      <c r="I57" s="70" t="s">
-        <v>98</v>
-      </c>
-      <c r="J57" s="70"/>
-      <c r="K57" s="71"/>
+      <c r="A57" s="137"/>
+      <c r="B57" s="138"/>
+      <c r="C57" s="138"/>
+      <c r="D57" s="138"/>
+      <c r="E57" s="125"/>
+      <c r="F57" s="125"/>
+      <c r="G57" s="169"/>
+      <c r="H57" s="169"/>
+      <c r="I57" s="125"/>
+      <c r="J57" s="125"/>
+      <c r="K57" s="127"/>
     </row>
     <row r="58" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="77"/>
-      <c r="B58" s="78"/>
-      <c r="C58" s="78"/>
-      <c r="D58" s="78"/>
-      <c r="E58" s="79"/>
-      <c r="F58" s="79"/>
-      <c r="G58" s="69"/>
-      <c r="H58" s="69"/>
-      <c r="I58" s="70"/>
-      <c r="J58" s="70"/>
-      <c r="K58" s="71"/>
+      <c r="A58" s="137"/>
+      <c r="B58" s="138"/>
+      <c r="C58" s="138"/>
+      <c r="D58" s="138"/>
+      <c r="E58" s="186"/>
+      <c r="F58" s="186"/>
+      <c r="G58" s="184"/>
+      <c r="H58" s="184"/>
+      <c r="I58" s="125"/>
+      <c r="J58" s="125"/>
+      <c r="K58" s="127"/>
     </row>
     <row r="59" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="72"/>
-      <c r="B59" s="73"/>
-      <c r="C59" s="73"/>
-      <c r="D59" s="73"/>
-      <c r="E59" s="73"/>
-      <c r="F59" s="73"/>
-      <c r="G59" s="74"/>
-      <c r="H59" s="74"/>
-      <c r="I59" s="75"/>
-      <c r="J59" s="75"/>
-      <c r="K59" s="76"/>
+      <c r="A59" s="139"/>
+      <c r="B59" s="140"/>
+      <c r="C59" s="140"/>
+      <c r="D59" s="140"/>
+      <c r="E59" s="140"/>
+      <c r="F59" s="140"/>
+      <c r="G59" s="185"/>
+      <c r="H59" s="185"/>
+      <c r="I59" s="145"/>
+      <c r="J59" s="145"/>
+      <c r="K59" s="146"/>
     </row>
     <row r="60" spans="1:11" s="1" customFormat="1" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="58" t="s">
+      <c r="A60" s="173" t="s">
         <v>82</v>
       </c>
-      <c r="B60" s="59"/>
-      <c r="C60" s="59"/>
-      <c r="D60" s="59"/>
-      <c r="E60" s="59"/>
-      <c r="F60" s="59"/>
-      <c r="G60" s="59"/>
-      <c r="H60" s="59"/>
-      <c r="I60" s="60"/>
-      <c r="J60" s="60"/>
-      <c r="K60" s="61"/>
+      <c r="B60" s="174"/>
+      <c r="C60" s="174"/>
+      <c r="D60" s="174"/>
+      <c r="E60" s="174"/>
+      <c r="F60" s="174"/>
+      <c r="G60" s="174"/>
+      <c r="H60" s="174"/>
+      <c r="I60" s="175"/>
+      <c r="J60" s="175"/>
+      <c r="K60" s="176"/>
     </row>
     <row r="61" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="65" t="s">
+      <c r="A61" s="180" t="s">
         <v>33</v>
       </c>
-      <c r="B61" s="66"/>
-      <c r="C61" s="67" t="s">
-        <v>137</v>
-      </c>
-      <c r="D61" s="67"/>
-      <c r="E61" s="67"/>
-      <c r="F61" s="67"/>
-      <c r="G61" s="67"/>
-      <c r="H61" s="67"/>
-      <c r="I61" s="67"/>
-      <c r="J61" s="67"/>
-      <c r="K61" s="68"/>
+      <c r="B61" s="181"/>
+      <c r="C61" s="182"/>
+      <c r="D61" s="182"/>
+      <c r="E61" s="182"/>
+      <c r="F61" s="182"/>
+      <c r="G61" s="182"/>
+      <c r="H61" s="182"/>
+      <c r="I61" s="182"/>
+      <c r="J61" s="182"/>
+      <c r="K61" s="183"/>
     </row>
     <row r="62" spans="1:11" s="1" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="22"/>
@@ -3748,20 +3663,20 @@
       <c r="K62" s="23"/>
     </row>
     <row r="63" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="62" t="s">
+      <c r="A63" s="177" t="s">
         <v>34</v>
       </c>
-      <c r="B63" s="63"/>
-      <c r="C63" s="63"/>
-      <c r="D63" s="63"/>
-      <c r="E63" s="63"/>
-      <c r="G63" s="63" t="s">
+      <c r="B63" s="178"/>
+      <c r="C63" s="178"/>
+      <c r="D63" s="178"/>
+      <c r="E63" s="178"/>
+      <c r="G63" s="178" t="s">
         <v>52</v>
       </c>
-      <c r="H63" s="63"/>
-      <c r="I63" s="63"/>
-      <c r="J63" s="63"/>
-      <c r="K63" s="64"/>
+      <c r="H63" s="178"/>
+      <c r="I63" s="178"/>
+      <c r="J63" s="178"/>
+      <c r="K63" s="179"/>
     </row>
     <row r="64" spans="1:11" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="24"/>
@@ -3778,6 +3693,123 @@
     </row>
   </sheetData>
   <mergeCells count="141">
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="G63:K63"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="C61:K61"/>
+    <mergeCell ref="G58:H58"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="G59:H59"/>
+    <mergeCell ref="I59:K59"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="J52:K52"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="A55:K55"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="G56:H56"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="A49:K49"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="J51:K51"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="J50:K50"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="J46:K46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="J47:K47"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="A38:K38"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="A28:K28"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="F29:K29"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="A32:K32"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="F30:K30"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A17:B18"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="I21:K21"/>
     <mergeCell ref="M8:V8"/>
     <mergeCell ref="M9:V9"/>
     <mergeCell ref="M10:V10"/>
@@ -3802,123 +3834,6 @@
     <mergeCell ref="E12:K12"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="E13:K13"/>
-    <mergeCell ref="A17:B18"/>
-    <mergeCell ref="A14:K14"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="A24:K24"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="A20:K20"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="A28:K28"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="F29:K29"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="A32:K32"/>
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="F30:K30"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A38:K38"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="J46:K46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="J47:K47"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="A49:K49"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="H51:I51"/>
-    <mergeCell ref="J51:K51"/>
-    <mergeCell ref="H50:I50"/>
-    <mergeCell ref="J50:K50"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="G57:H57"/>
-    <mergeCell ref="H52:I52"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="J52:K52"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="A55:K55"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="G56:H56"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="A60:H60"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="A63:E63"/>
-    <mergeCell ref="G63:K63"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="C61:K61"/>
-    <mergeCell ref="G58:H58"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="G59:H59"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="E58:F58"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -3960,41 +3875,41 @@
     </row>
     <row r="2" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="32"/>
-      <c r="D2" s="155" t="s">
+      <c r="D2" s="67" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="155"/>
-      <c r="F2" s="155"/>
-      <c r="G2" s="155"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="155"/>
-      <c r="J2" s="155"/>
-      <c r="K2" s="156"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="32"/>
-      <c r="D3" s="155"/>
-      <c r="E3" s="155"/>
-      <c r="F3" s="155"/>
-      <c r="G3" s="155"/>
-      <c r="H3" s="155"/>
-      <c r="I3" s="155"/>
-      <c r="J3" s="155"/>
-      <c r="K3" s="156"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="68"/>
     </row>
     <row r="4" spans="1:11" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
       <c r="B4" s="25"/>
       <c r="C4" s="25"/>
-      <c r="D4" s="187" t="s">
+      <c r="D4" s="238" t="s">
         <v>84</v>
       </c>
-      <c r="E4" s="187"/>
-      <c r="F4" s="187"/>
-      <c r="G4" s="187"/>
-      <c r="H4" s="187"/>
-      <c r="I4" s="187"/>
-      <c r="J4" s="187"/>
+      <c r="E4" s="238"/>
+      <c r="F4" s="238"/>
+      <c r="G4" s="238"/>
+      <c r="H4" s="238"/>
+      <c r="I4" s="238"/>
+      <c r="J4" s="238"/>
       <c r="K4" s="34" t="s">
         <v>83</v>
       </c>
@@ -4011,57 +3926,53 @@
       <c r="K5" s="23"/>
     </row>
     <row r="6" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="195" t="s">
+      <c r="A6" s="243" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="196"/>
-      <c r="C6" s="196"/>
-      <c r="D6" s="196"/>
-      <c r="E6" s="196"/>
-      <c r="F6" s="196"/>
-      <c r="G6" s="196"/>
-      <c r="H6" s="196"/>
-      <c r="I6" s="196"/>
-      <c r="J6" s="196"/>
-      <c r="K6" s="197"/>
+      <c r="B6" s="244"/>
+      <c r="C6" s="244"/>
+      <c r="D6" s="244"/>
+      <c r="E6" s="244"/>
+      <c r="F6" s="244"/>
+      <c r="G6" s="244"/>
+      <c r="H6" s="244"/>
+      <c r="I6" s="244"/>
+      <c r="J6" s="244"/>
+      <c r="K6" s="245"/>
     </row>
     <row r="7" spans="1:11" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="182" t="s">
+      <c r="A7" s="94" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="183"/>
-      <c r="C7" s="183"/>
-      <c r="D7" s="183"/>
-      <c r="E7" s="198" t="s">
-        <v>138</v>
-      </c>
-      <c r="F7" s="199"/>
-      <c r="G7" s="199"/>
-      <c r="H7" s="199"/>
-      <c r="I7" s="199"/>
-      <c r="J7" s="199"/>
-      <c r="K7" s="200"/>
+      <c r="B7" s="95"/>
+      <c r="C7" s="95"/>
+      <c r="D7" s="95"/>
+      <c r="E7" s="246"/>
+      <c r="F7" s="247"/>
+      <c r="G7" s="247"/>
+      <c r="H7" s="247"/>
+      <c r="I7" s="247"/>
+      <c r="J7" s="247"/>
+      <c r="K7" s="248"/>
     </row>
     <row r="8" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="182" t="s">
+      <c r="A8" s="94" t="s">
         <v>58</v>
       </c>
-      <c r="B8" s="183"/>
-      <c r="C8" s="183"/>
-      <c r="D8" s="183"/>
-      <c r="E8" s="201" t="s">
-        <v>139</v>
-      </c>
-      <c r="F8" s="202"/>
-      <c r="G8" s="202"/>
-      <c r="H8" s="202"/>
-      <c r="I8" s="202"/>
-      <c r="J8" s="202"/>
-      <c r="K8" s="203"/>
+      <c r="B8" s="95"/>
+      <c r="C8" s="95"/>
+      <c r="D8" s="95"/>
+      <c r="E8" s="249"/>
+      <c r="F8" s="250"/>
+      <c r="G8" s="250"/>
+      <c r="H8" s="250"/>
+      <c r="I8" s="250"/>
+      <c r="J8" s="250"/>
+      <c r="K8" s="251"/>
     </row>
     <row r="9" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="57" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="B9" s="37"/>
       <c r="C9" s="37"/>
@@ -4081,9 +3992,7 @@
       <c r="B10" s="36"/>
       <c r="C10" s="36"/>
       <c r="D10" s="36"/>
-      <c r="E10" s="20" t="s">
-        <v>86</v>
-      </c>
+      <c r="E10" s="20"/>
       <c r="F10" s="20"/>
       <c r="G10" s="20"/>
       <c r="H10" s="20"/>
@@ -4105,286 +4014,266 @@
       <c r="K11" s="42"/>
     </row>
     <row r="12" spans="1:11" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="207" t="s">
+      <c r="A12" s="205" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="208"/>
-      <c r="C12" s="208"/>
-      <c r="D12" s="208"/>
-      <c r="E12" s="208"/>
-      <c r="F12" s="208"/>
-      <c r="G12" s="208"/>
-      <c r="H12" s="208"/>
-      <c r="I12" s="208"/>
-      <c r="J12" s="208"/>
-      <c r="K12" s="209"/>
+      <c r="B12" s="206"/>
+      <c r="C12" s="206"/>
+      <c r="D12" s="206"/>
+      <c r="E12" s="206"/>
+      <c r="F12" s="206"/>
+      <c r="G12" s="206"/>
+      <c r="H12" s="206"/>
+      <c r="I12" s="206"/>
+      <c r="J12" s="206"/>
+      <c r="K12" s="207"/>
     </row>
     <row r="13" spans="1:11" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="210" t="s">
+      <c r="A13" s="203" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="211"/>
-      <c r="C13" s="211" t="s">
+      <c r="B13" s="204"/>
+      <c r="C13" s="204" t="s">
         <v>61</v>
       </c>
-      <c r="D13" s="211"/>
-      <c r="E13" s="211"/>
-      <c r="F13" s="211"/>
-      <c r="G13" s="211" t="s">
+      <c r="D13" s="204"/>
+      <c r="E13" s="204"/>
+      <c r="F13" s="204"/>
+      <c r="G13" s="204" t="s">
         <v>60</v>
       </c>
-      <c r="H13" s="211"/>
-      <c r="I13" s="211"/>
-      <c r="J13" s="211"/>
-      <c r="K13" s="255"/>
+      <c r="H13" s="204"/>
+      <c r="I13" s="204"/>
+      <c r="J13" s="204"/>
+      <c r="K13" s="208"/>
     </row>
     <row r="14" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="179" t="s">
+      <c r="A14" s="91" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="242"/>
-      <c r="C14" s="194">
-        <v>39</v>
-      </c>
-      <c r="D14" s="194"/>
-      <c r="E14" s="194"/>
-      <c r="F14" s="194"/>
-      <c r="G14" s="194"/>
-      <c r="H14" s="194"/>
-      <c r="I14" s="194"/>
-      <c r="J14" s="194"/>
-      <c r="K14" s="253"/>
+      <c r="B14" s="193"/>
+      <c r="C14" s="199"/>
+      <c r="D14" s="199"/>
+      <c r="E14" s="199"/>
+      <c r="F14" s="199"/>
+      <c r="G14" s="199"/>
+      <c r="H14" s="199"/>
+      <c r="I14" s="199"/>
+      <c r="J14" s="199"/>
+      <c r="K14" s="200"/>
     </row>
     <row r="15" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="179" t="s">
+      <c r="A15" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="242"/>
-      <c r="C15" s="194">
-        <v>39</v>
-      </c>
-      <c r="D15" s="194"/>
-      <c r="E15" s="194"/>
-      <c r="F15" s="194"/>
-      <c r="G15" s="194"/>
-      <c r="H15" s="194"/>
-      <c r="I15" s="194"/>
-      <c r="J15" s="194"/>
-      <c r="K15" s="253"/>
+      <c r="B15" s="193"/>
+      <c r="C15" s="199"/>
+      <c r="D15" s="199"/>
+      <c r="E15" s="199"/>
+      <c r="F15" s="199"/>
+      <c r="G15" s="199"/>
+      <c r="H15" s="199"/>
+      <c r="I15" s="199"/>
+      <c r="J15" s="199"/>
+      <c r="K15" s="200"/>
     </row>
     <row r="16" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="248" t="s">
+      <c r="A16" s="194" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="249"/>
-      <c r="C16" s="252">
-        <v>38</v>
-      </c>
-      <c r="D16" s="252"/>
-      <c r="E16" s="252"/>
-      <c r="F16" s="252"/>
-      <c r="G16" s="252"/>
-      <c r="H16" s="252"/>
-      <c r="I16" s="252"/>
-      <c r="J16" s="252"/>
-      <c r="K16" s="254"/>
+      <c r="B16" s="195"/>
+      <c r="C16" s="198"/>
+      <c r="D16" s="198"/>
+      <c r="E16" s="198"/>
+      <c r="F16" s="198"/>
+      <c r="G16" s="198"/>
+      <c r="H16" s="198"/>
+      <c r="I16" s="198"/>
+      <c r="J16" s="198"/>
+      <c r="K16" s="201"/>
     </row>
     <row r="17" spans="1:11" s="7" customFormat="1" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="43"/>
       <c r="K17" s="44"/>
     </row>
     <row r="18" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="207" t="s">
+      <c r="A18" s="205" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="208"/>
-      <c r="C18" s="208"/>
-      <c r="D18" s="208"/>
-      <c r="E18" s="208"/>
-      <c r="F18" s="208"/>
-      <c r="G18" s="208"/>
-      <c r="H18" s="208"/>
-      <c r="I18" s="208"/>
-      <c r="J18" s="208"/>
-      <c r="K18" s="209"/>
+      <c r="B18" s="206"/>
+      <c r="C18" s="206"/>
+      <c r="D18" s="206"/>
+      <c r="E18" s="206"/>
+      <c r="F18" s="206"/>
+      <c r="G18" s="206"/>
+      <c r="H18" s="206"/>
+      <c r="I18" s="206"/>
+      <c r="J18" s="206"/>
+      <c r="K18" s="207"/>
     </row>
     <row r="19" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="210" t="s">
+      <c r="A19" s="203" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="211"/>
-      <c r="C19" s="250" t="s">
+      <c r="B19" s="204"/>
+      <c r="C19" s="196" t="s">
         <v>65</v>
       </c>
-      <c r="D19" s="250"/>
-      <c r="E19" s="250"/>
-      <c r="F19" s="250"/>
-      <c r="G19" s="250"/>
-      <c r="H19" s="250"/>
-      <c r="I19" s="250"/>
-      <c r="J19" s="250"/>
-      <c r="K19" s="251"/>
+      <c r="D19" s="196"/>
+      <c r="E19" s="196"/>
+      <c r="F19" s="196"/>
+      <c r="G19" s="196"/>
+      <c r="H19" s="196"/>
+      <c r="I19" s="196"/>
+      <c r="J19" s="196"/>
+      <c r="K19" s="197"/>
     </row>
     <row r="20" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="182" t="s">
+      <c r="A20" s="94" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="183"/>
-      <c r="C20" s="244" t="s">
-        <v>87</v>
-      </c>
-      <c r="D20" s="244"/>
-      <c r="E20" s="244"/>
-      <c r="F20" s="244"/>
-      <c r="G20" s="244"/>
-      <c r="H20" s="244"/>
-      <c r="I20" s="244"/>
-      <c r="J20" s="244"/>
-      <c r="K20" s="212" t="s">
+      <c r="B20" s="95"/>
+      <c r="C20" s="202"/>
+      <c r="D20" s="202"/>
+      <c r="E20" s="202"/>
+      <c r="F20" s="202"/>
+      <c r="G20" s="202"/>
+      <c r="H20" s="202"/>
+      <c r="I20" s="202"/>
+      <c r="J20" s="202"/>
+      <c r="K20" s="253" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="182" t="s">
+      <c r="A21" s="94" t="s">
         <v>63</v>
       </c>
-      <c r="B21" s="183"/>
-      <c r="C21" s="244" t="s">
-        <v>87</v>
-      </c>
-      <c r="D21" s="244"/>
-      <c r="E21" s="244"/>
-      <c r="F21" s="244"/>
-      <c r="G21" s="244"/>
-      <c r="H21" s="244"/>
-      <c r="I21" s="244"/>
-      <c r="J21" s="244"/>
-      <c r="K21" s="213"/>
+      <c r="B21" s="95"/>
+      <c r="C21" s="202"/>
+      <c r="D21" s="202"/>
+      <c r="E21" s="202"/>
+      <c r="F21" s="202"/>
+      <c r="G21" s="202"/>
+      <c r="H21" s="202"/>
+      <c r="I21" s="202"/>
+      <c r="J21" s="202"/>
+      <c r="K21" s="254"/>
     </row>
     <row r="22" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="243"/>
-      <c r="B22" s="193"/>
-      <c r="C22" s="244"/>
-      <c r="D22" s="244"/>
-      <c r="E22" s="244"/>
-      <c r="F22" s="244"/>
-      <c r="G22" s="244"/>
-      <c r="H22" s="244"/>
-      <c r="I22" s="244"/>
-      <c r="J22" s="244"/>
-      <c r="K22" s="214"/>
+      <c r="A22" s="210"/>
+      <c r="B22" s="211"/>
+      <c r="C22" s="202"/>
+      <c r="D22" s="202"/>
+      <c r="E22" s="202"/>
+      <c r="F22" s="202"/>
+      <c r="G22" s="202"/>
+      <c r="H22" s="202"/>
+      <c r="I22" s="202"/>
+      <c r="J22" s="202"/>
+      <c r="K22" s="255"/>
     </row>
     <row r="23" spans="1:11" s="1" customFormat="1" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="45"/>
       <c r="K23" s="46"/>
     </row>
     <row r="24" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="117" t="s">
+      <c r="A24" s="128" t="s">
         <v>66</v>
       </c>
-      <c r="B24" s="205"/>
-      <c r="C24" s="205"/>
-      <c r="D24" s="118"/>
-      <c r="E24" s="204" t="s">
+      <c r="B24" s="209"/>
+      <c r="C24" s="209"/>
+      <c r="D24" s="129"/>
+      <c r="E24" s="212" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="205"/>
-      <c r="G24" s="118"/>
-      <c r="H24" s="204" t="s">
+      <c r="F24" s="209"/>
+      <c r="G24" s="129"/>
+      <c r="H24" s="212" t="s">
         <v>40</v>
       </c>
-      <c r="I24" s="205"/>
-      <c r="J24" s="205"/>
-      <c r="K24" s="206"/>
+      <c r="I24" s="209"/>
+      <c r="J24" s="209"/>
+      <c r="K24" s="252"/>
     </row>
     <row r="25" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="217" t="s">
+      <c r="A25" s="227" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="218"/>
-      <c r="C25" s="188" t="s">
+      <c r="B25" s="228"/>
+      <c r="C25" s="218" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="188"/>
-      <c r="E25" s="79" t="s">
-        <v>99</v>
-      </c>
-      <c r="F25" s="79"/>
-      <c r="G25" s="79"/>
-      <c r="H25" s="223" t="s">
-        <v>95</v>
-      </c>
-      <c r="I25" s="224"/>
-      <c r="J25" s="224"/>
-      <c r="K25" s="233"/>
+      <c r="D25" s="218"/>
+      <c r="E25" s="186"/>
+      <c r="F25" s="186"/>
+      <c r="G25" s="186"/>
+      <c r="H25" s="213"/>
+      <c r="I25" s="214"/>
+      <c r="J25" s="214"/>
+      <c r="K25" s="215"/>
     </row>
     <row r="26" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="219"/>
-      <c r="B26" s="220"/>
-      <c r="C26" s="188" t="s">
+      <c r="A26" s="229"/>
+      <c r="B26" s="230"/>
+      <c r="C26" s="218" t="s">
         <v>50</v>
       </c>
-      <c r="D26" s="188"/>
-      <c r="E26" s="223">
-        <v>226784</v>
-      </c>
-      <c r="F26" s="224"/>
-      <c r="G26" s="225"/>
-      <c r="H26" s="223">
-        <v>6823</v>
-      </c>
-      <c r="I26" s="224"/>
-      <c r="J26" s="224"/>
-      <c r="K26" s="233"/>
+      <c r="D26" s="218"/>
+      <c r="E26" s="213"/>
+      <c r="F26" s="214"/>
+      <c r="G26" s="233"/>
+      <c r="H26" s="213"/>
+      <c r="I26" s="214"/>
+      <c r="J26" s="214"/>
+      <c r="K26" s="215"/>
     </row>
     <row r="27" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="221"/>
-      <c r="B27" s="222"/>
-      <c r="C27" s="188" t="s">
+      <c r="A27" s="231"/>
+      <c r="B27" s="232"/>
+      <c r="C27" s="218" t="s">
         <v>42</v>
       </c>
-      <c r="D27" s="188"/>
-      <c r="E27" s="70"/>
-      <c r="F27" s="70"/>
-      <c r="G27" s="70"/>
-      <c r="H27" s="78"/>
-      <c r="I27" s="78"/>
-      <c r="J27" s="78"/>
-      <c r="K27" s="234"/>
+      <c r="D27" s="218"/>
+      <c r="E27" s="125"/>
+      <c r="F27" s="125"/>
+      <c r="G27" s="125"/>
+      <c r="H27" s="138"/>
+      <c r="I27" s="138"/>
+      <c r="J27" s="138"/>
+      <c r="K27" s="216"/>
     </row>
     <row r="28" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="189" t="s">
+      <c r="A28" s="239" t="s">
         <v>43</v>
       </c>
-      <c r="B28" s="190"/>
-      <c r="C28" s="183" t="s">
+      <c r="B28" s="240"/>
+      <c r="C28" s="95" t="s">
         <v>41</v>
       </c>
-      <c r="D28" s="183"/>
-      <c r="E28" s="79"/>
-      <c r="F28" s="79"/>
-      <c r="G28" s="79"/>
-      <c r="H28" s="223" t="s">
-        <v>90</v>
-      </c>
-      <c r="I28" s="224"/>
-      <c r="J28" s="224"/>
-      <c r="K28" s="233"/>
+      <c r="D28" s="95"/>
+      <c r="E28" s="186"/>
+      <c r="F28" s="186"/>
+      <c r="G28" s="186"/>
+      <c r="H28" s="213"/>
+      <c r="I28" s="214"/>
+      <c r="J28" s="214"/>
+      <c r="K28" s="215"/>
     </row>
     <row r="29" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="191"/>
-      <c r="B29" s="192"/>
-      <c r="C29" s="193" t="s">
+      <c r="A29" s="241"/>
+      <c r="B29" s="242"/>
+      <c r="C29" s="211" t="s">
         <v>42</v>
       </c>
-      <c r="D29" s="193"/>
-      <c r="E29" s="215"/>
-      <c r="F29" s="215"/>
-      <c r="G29" s="215"/>
-      <c r="H29" s="73"/>
-      <c r="I29" s="73"/>
-      <c r="J29" s="73"/>
-      <c r="K29" s="235"/>
+      <c r="D29" s="211"/>
+      <c r="E29" s="225"/>
+      <c r="F29" s="225"/>
+      <c r="G29" s="225"/>
+      <c r="H29" s="140"/>
+      <c r="I29" s="140"/>
+      <c r="J29" s="140"/>
+      <c r="K29" s="217"/>
     </row>
     <row r="30" spans="1:11" s="1" customFormat="1" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="47"/>
@@ -4400,249 +4289,299 @@
       <c r="K30" s="48"/>
     </row>
     <row r="31" spans="1:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="173" t="s">
+      <c r="A31" s="85" t="s">
         <v>51</v>
       </c>
-      <c r="B31" s="174"/>
-      <c r="C31" s="174"/>
-      <c r="D31" s="174"/>
-      <c r="E31" s="174"/>
-      <c r="F31" s="174"/>
-      <c r="G31" s="174"/>
-      <c r="H31" s="174"/>
-      <c r="I31" s="174"/>
-      <c r="J31" s="174"/>
-      <c r="K31" s="175"/>
+      <c r="B31" s="86"/>
+      <c r="C31" s="86"/>
+      <c r="D31" s="86"/>
+      <c r="E31" s="86"/>
+      <c r="F31" s="86"/>
+      <c r="G31" s="86"/>
+      <c r="H31" s="86"/>
+      <c r="I31" s="86"/>
+      <c r="J31" s="86"/>
+      <c r="K31" s="87"/>
     </row>
     <row r="32" spans="1:11" s="14" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="216" t="s">
+      <c r="A32" s="226" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="184"/>
-      <c r="C32" s="184"/>
-      <c r="D32" s="184"/>
-      <c r="E32" s="184"/>
-      <c r="F32" s="184"/>
-      <c r="G32" s="184"/>
-      <c r="H32" s="184"/>
-      <c r="I32" s="184"/>
-      <c r="J32" s="184"/>
-      <c r="K32" s="185"/>
+      <c r="B32" s="96"/>
+      <c r="C32" s="96"/>
+      <c r="D32" s="96"/>
+      <c r="E32" s="96"/>
+      <c r="F32" s="96"/>
+      <c r="G32" s="96"/>
+      <c r="H32" s="96"/>
+      <c r="I32" s="96"/>
+      <c r="J32" s="96"/>
+      <c r="K32" s="97"/>
     </row>
     <row r="33" spans="1:11" s="14" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="182" t="s">
+      <c r="A33" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="183"/>
-      <c r="C33" s="183"/>
-      <c r="D33" s="183"/>
-      <c r="E33" s="183"/>
-      <c r="F33" s="183"/>
-      <c r="G33" s="183"/>
-      <c r="H33" s="183"/>
-      <c r="I33" s="183"/>
-      <c r="J33" s="183"/>
-      <c r="K33" s="186"/>
+      <c r="B33" s="95"/>
+      <c r="C33" s="95"/>
+      <c r="D33" s="95"/>
+      <c r="E33" s="95"/>
+      <c r="F33" s="95"/>
+      <c r="G33" s="95"/>
+      <c r="H33" s="95"/>
+      <c r="I33" s="95"/>
+      <c r="J33" s="95"/>
+      <c r="K33" s="98"/>
     </row>
     <row r="34" spans="1:11" s="1" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="226" t="s">
-        <v>88</v>
-      </c>
-      <c r="B34" s="227"/>
-      <c r="C34" s="228"/>
-      <c r="D34" s="226" t="s">
-        <v>89</v>
-      </c>
-      <c r="E34" s="227"/>
-      <c r="F34" s="227"/>
-      <c r="G34" s="228"/>
-      <c r="H34" s="226" t="s">
-        <v>96</v>
-      </c>
-      <c r="I34" s="227"/>
-      <c r="J34" s="227"/>
-      <c r="K34" s="229"/>
+      <c r="A34" s="234" t="s">
+        <v>85</v>
+      </c>
+      <c r="B34" s="235"/>
+      <c r="C34" s="236"/>
+      <c r="D34" s="234" t="s">
+        <v>86</v>
+      </c>
+      <c r="E34" s="235"/>
+      <c r="F34" s="235"/>
+      <c r="G34" s="236"/>
+      <c r="H34" s="234" t="s">
+        <v>90</v>
+      </c>
+      <c r="I34" s="235"/>
+      <c r="J34" s="235"/>
+      <c r="K34" s="237"/>
     </row>
     <row r="35" spans="1:11" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="182" t="s">
+      <c r="A35" s="94" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="183"/>
-      <c r="C35" s="183"/>
-      <c r="D35" s="239">
-        <v>9000</v>
-      </c>
-      <c r="E35" s="240"/>
-      <c r="F35" s="240"/>
-      <c r="G35" s="240"/>
-      <c r="H35" s="240"/>
-      <c r="I35" s="240"/>
-      <c r="J35" s="240"/>
-      <c r="K35" s="241"/>
+      <c r="B35" s="95"/>
+      <c r="C35" s="95"/>
+      <c r="D35" s="222"/>
+      <c r="E35" s="223"/>
+      <c r="F35" s="223"/>
+      <c r="G35" s="223"/>
+      <c r="H35" s="223"/>
+      <c r="I35" s="223"/>
+      <c r="J35" s="223"/>
+      <c r="K35" s="224"/>
     </row>
     <row r="36" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="182" t="s">
+      <c r="A36" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="183"/>
-      <c r="C36" s="183"/>
-      <c r="D36" s="183"/>
-      <c r="E36" s="183"/>
-      <c r="F36" s="183"/>
-      <c r="G36" s="183"/>
-      <c r="H36" s="183"/>
-      <c r="I36" s="183"/>
-      <c r="J36" s="183"/>
-      <c r="K36" s="186"/>
+      <c r="B36" s="95"/>
+      <c r="C36" s="95"/>
+      <c r="D36" s="95"/>
+      <c r="E36" s="95"/>
+      <c r="F36" s="95"/>
+      <c r="G36" s="95"/>
+      <c r="H36" s="95"/>
+      <c r="I36" s="95"/>
+      <c r="J36" s="95"/>
+      <c r="K36" s="98"/>
     </row>
     <row r="37" spans="1:11" s="19" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="182" t="s">
+      <c r="A37" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="B37" s="183"/>
-      <c r="C37" s="183"/>
-      <c r="D37" s="183"/>
-      <c r="E37" s="183"/>
-      <c r="F37" s="183"/>
-      <c r="G37" s="183"/>
-      <c r="H37" s="183"/>
-      <c r="I37" s="183"/>
-      <c r="J37" s="183"/>
-      <c r="K37" s="186"/>
+      <c r="B37" s="95"/>
+      <c r="C37" s="95"/>
+      <c r="D37" s="95"/>
+      <c r="E37" s="95"/>
+      <c r="F37" s="95"/>
+      <c r="G37" s="95"/>
+      <c r="H37" s="95"/>
+      <c r="I37" s="95"/>
+      <c r="J37" s="95"/>
+      <c r="K37" s="98"/>
     </row>
     <row r="38" spans="1:11" s="19" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="182" t="s">
+      <c r="A38" s="94" t="s">
         <v>16</v>
       </c>
-      <c r="B38" s="183"/>
-      <c r="C38" s="183"/>
-      <c r="D38" s="183"/>
-      <c r="E38" s="183"/>
-      <c r="F38" s="183"/>
-      <c r="G38" s="183"/>
-      <c r="H38" s="183"/>
-      <c r="I38" s="183"/>
-      <c r="J38" s="183"/>
-      <c r="K38" s="186"/>
+      <c r="B38" s="95"/>
+      <c r="C38" s="95"/>
+      <c r="D38" s="95"/>
+      <c r="E38" s="95"/>
+      <c r="F38" s="95"/>
+      <c r="G38" s="95"/>
+      <c r="H38" s="95"/>
+      <c r="I38" s="95"/>
+      <c r="J38" s="95"/>
+      <c r="K38" s="98"/>
     </row>
     <row r="39" spans="1:11" s="19" customFormat="1" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="182" t="s">
+      <c r="A39" s="94" t="s">
         <v>17</v>
       </c>
-      <c r="B39" s="183"/>
-      <c r="C39" s="183"/>
-      <c r="D39" s="183"/>
-      <c r="E39" s="183"/>
-      <c r="F39" s="183"/>
-      <c r="G39" s="183"/>
-      <c r="H39" s="183"/>
-      <c r="I39" s="183"/>
-      <c r="J39" s="183"/>
-      <c r="K39" s="186"/>
+      <c r="B39" s="95"/>
+      <c r="C39" s="95"/>
+      <c r="D39" s="95"/>
+      <c r="E39" s="95"/>
+      <c r="F39" s="95"/>
+      <c r="G39" s="95"/>
+      <c r="H39" s="95"/>
+      <c r="I39" s="95"/>
+      <c r="J39" s="95"/>
+      <c r="K39" s="98"/>
     </row>
     <row r="40" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="236" t="s">
+      <c r="A40" s="219" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="237"/>
-      <c r="C40" s="237"/>
-      <c r="D40" s="237"/>
-      <c r="E40" s="237"/>
-      <c r="F40" s="237"/>
-      <c r="G40" s="237"/>
-      <c r="H40" s="237"/>
-      <c r="I40" s="237"/>
-      <c r="J40" s="237"/>
-      <c r="K40" s="238"/>
+      <c r="B40" s="220"/>
+      <c r="C40" s="220"/>
+      <c r="D40" s="220"/>
+      <c r="E40" s="220"/>
+      <c r="F40" s="220"/>
+      <c r="G40" s="220"/>
+      <c r="H40" s="220"/>
+      <c r="I40" s="220"/>
+      <c r="J40" s="220"/>
+      <c r="K40" s="221"/>
     </row>
     <row r="41" spans="1:11" s="1" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="230" t="s">
-        <v>106</v>
-      </c>
-      <c r="B41" s="231"/>
-      <c r="C41" s="231"/>
-      <c r="D41" s="231"/>
-      <c r="E41" s="231"/>
-      <c r="F41" s="231"/>
-      <c r="G41" s="231"/>
-      <c r="H41" s="231"/>
-      <c r="I41" s="231"/>
-      <c r="J41" s="231"/>
-      <c r="K41" s="232"/>
+      <c r="A41" s="187" t="s">
+        <v>98</v>
+      </c>
+      <c r="B41" s="188"/>
+      <c r="C41" s="188"/>
+      <c r="D41" s="188"/>
+      <c r="E41" s="188"/>
+      <c r="F41" s="188"/>
+      <c r="G41" s="188"/>
+      <c r="H41" s="188"/>
+      <c r="I41" s="188"/>
+      <c r="J41" s="188"/>
+      <c r="K41" s="189"/>
     </row>
     <row r="42" spans="1:11" s="1" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="230" t="s">
-        <v>94</v>
-      </c>
-      <c r="B42" s="231"/>
-      <c r="C42" s="231"/>
-      <c r="D42" s="231"/>
-      <c r="E42" s="231"/>
-      <c r="F42" s="231"/>
-      <c r="G42" s="231"/>
-      <c r="H42" s="231"/>
-      <c r="I42" s="231"/>
-      <c r="J42" s="231"/>
-      <c r="K42" s="232"/>
+      <c r="A42" s="187" t="s">
+        <v>115</v>
+      </c>
+      <c r="B42" s="188"/>
+      <c r="C42" s="188"/>
+      <c r="D42" s="188"/>
+      <c r="E42" s="188"/>
+      <c r="F42" s="188"/>
+      <c r="G42" s="188"/>
+      <c r="H42" s="188"/>
+      <c r="I42" s="188"/>
+      <c r="J42" s="188"/>
+      <c r="K42" s="189"/>
     </row>
     <row r="43" spans="1:11" s="1" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="230" t="s">
-        <v>92</v>
-      </c>
-      <c r="B43" s="231"/>
-      <c r="C43" s="231"/>
-      <c r="D43" s="231"/>
-      <c r="E43" s="231"/>
-      <c r="F43" s="231"/>
-      <c r="G43" s="231"/>
-      <c r="H43" s="231"/>
-      <c r="I43" s="231"/>
-      <c r="J43" s="231"/>
-      <c r="K43" s="232"/>
+      <c r="A43" s="187" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" s="188"/>
+      <c r="C43" s="188"/>
+      <c r="D43" s="188"/>
+      <c r="E43" s="188"/>
+      <c r="F43" s="188"/>
+      <c r="G43" s="188"/>
+      <c r="H43" s="188"/>
+      <c r="I43" s="188"/>
+      <c r="J43" s="188"/>
+      <c r="K43" s="189"/>
     </row>
     <row r="44" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="230"/>
-      <c r="B44" s="231"/>
-      <c r="C44" s="231"/>
-      <c r="D44" s="231"/>
-      <c r="E44" s="231"/>
-      <c r="F44" s="231"/>
-      <c r="G44" s="231"/>
-      <c r="H44" s="231"/>
-      <c r="I44" s="231"/>
-      <c r="J44" s="231"/>
-      <c r="K44" s="232"/>
+      <c r="A44" s="187"/>
+      <c r="B44" s="188"/>
+      <c r="C44" s="188"/>
+      <c r="D44" s="188"/>
+      <c r="E44" s="188"/>
+      <c r="F44" s="188"/>
+      <c r="G44" s="188"/>
+      <c r="H44" s="188"/>
+      <c r="I44" s="188"/>
+      <c r="J44" s="188"/>
+      <c r="K44" s="189"/>
     </row>
     <row r="45" spans="1:11" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="245"/>
-      <c r="B45" s="246"/>
-      <c r="C45" s="246"/>
-      <c r="D45" s="246"/>
-      <c r="E45" s="246"/>
-      <c r="F45" s="246"/>
-      <c r="G45" s="246"/>
-      <c r="H45" s="246"/>
-      <c r="I45" s="246"/>
-      <c r="J45" s="246"/>
-      <c r="K45" s="247"/>
+      <c r="A45" s="190"/>
+      <c r="B45" s="191"/>
+      <c r="C45" s="191"/>
+      <c r="D45" s="191"/>
+      <c r="E45" s="191"/>
+      <c r="F45" s="191"/>
+      <c r="G45" s="191"/>
+      <c r="H45" s="191"/>
+      <c r="I45" s="191"/>
+      <c r="J45" s="191"/>
+      <c r="K45" s="192"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="68">
+    <mergeCell ref="D4:J4"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="A31:K31"/>
+    <mergeCell ref="A28:B29"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="E7:K7"/>
+    <mergeCell ref="E8:K8"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="K20:K22"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A33:K33"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="A32:K32"/>
+    <mergeCell ref="A25:B27"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D34:G34"/>
+    <mergeCell ref="H34:K34"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="H27:K27"/>
+    <mergeCell ref="H28:K28"/>
+    <mergeCell ref="H29:K29"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A40:K40"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="D35:K35"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A38:K38"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="H26:K26"/>
+    <mergeCell ref="A39:K39"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C21:J21"/>
+    <mergeCell ref="C22:J22"/>
+    <mergeCell ref="E24:G24"/>
     <mergeCell ref="A44:K44"/>
     <mergeCell ref="A45:K45"/>
     <mergeCell ref="D2:K3"/>
@@ -4659,58 +4598,6 @@
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="G13:K13"/>
     <mergeCell ref="C13:F13"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C21:J21"/>
-    <mergeCell ref="C22:J22"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="A43:K43"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="H27:K27"/>
-    <mergeCell ref="H28:K28"/>
-    <mergeCell ref="H29:K29"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A40:K40"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="D35:K35"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A38:K38"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="A37:K37"/>
-    <mergeCell ref="H26:K26"/>
-    <mergeCell ref="A39:K39"/>
-    <mergeCell ref="A36:K36"/>
-    <mergeCell ref="A33:K33"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="A32:K32"/>
-    <mergeCell ref="A25:B27"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:G34"/>
-    <mergeCell ref="H34:K34"/>
-    <mergeCell ref="D4:J4"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="A31:K31"/>
-    <mergeCell ref="A28:B29"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="A6:K6"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="E7:K7"/>
-    <mergeCell ref="E8:K8"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="A12:K12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="K20:K22"/>
-    <mergeCell ref="C15:F15"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Atualização regras 1004 v2
</commit_message>
<xml_diff>
--- a/backend/assets/template_supra.xlsx
+++ b/backend/assets/template_supra.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projeto Sistema pedidos\Planejamento\Arquivos bases edson\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\OrderSync\backend\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAEC6108-A469-4EE7-A5AC-A7F4E92CE825}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A66C742-6B4B-426B-BC49-BAA751F763A1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cadastro Parte 1" sheetId="5" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="117">
   <si>
     <t>COMERCIAL</t>
   </si>
@@ -339,9 +339,6 @@
     <t xml:space="preserve">    Lojista = (Produto para Comercializar / Revender)</t>
   </si>
   <si>
-    <t xml:space="preserve">      (XX)Cobrança      </t>
-  </si>
-  <si>
     <t xml:space="preserve">CPF:    </t>
   </si>
   <si>
@@ -372,9 +369,6 @@
     <t xml:space="preserve">Cli Direto:      </t>
   </si>
   <si>
-    <t>Utilização do Produto:   (   )Insumos na Pecuária   (   )Consumo Próprio   (   )Industrialização   (XX)Comercializar/Revender</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nome do Cliente:  </t>
   </si>
   <si>
@@ -415,6 +409,15 @@
   </si>
   <si>
     <t>Lojista = (Produto para Comercializar / Revender)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      ( )Cobrança      </t>
+  </si>
+  <si>
+    <t>DISPET REPRESENTAÇÕES COMERCIAIS - CÓDIGO 178799</t>
+  </si>
+  <si>
+    <t>Utilização do Produto:   (   )Insumos na Pecuária   (   )Consumo Próprio   (   )Industrialização   ( )Comercializar/Revender</t>
   </si>
 </sst>
 </file>
@@ -425,7 +428,7 @@
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00;[Red]&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -514,27 +517,13 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF002060"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -547,12 +536,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="53">
     <border>
@@ -1194,7 +1177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="256">
+  <cellXfs count="247">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1341,32 +1324,269 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1464,383 +1684,89 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1866,6 +1792,12 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1881,59 +1813,83 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2646,7 +2602,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V64"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="10" width="9.7109375" customWidth="1"/>
@@ -2654,7 +2610,7 @@
     <col min="12" max="12" width="5.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="29"/>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -2667,31 +2623,31 @@
       <c r="J1" s="30"/>
       <c r="K1" s="31"/>
     </row>
-    <row r="2" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="32"/>
-      <c r="D2" s="67" t="s">
+      <c r="D2" s="146" t="s">
         <v>80</v>
       </c>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
-    </row>
-    <row r="3" spans="1:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E2" s="146"/>
+      <c r="F2" s="146"/>
+      <c r="G2" s="146"/>
+      <c r="H2" s="146"/>
+      <c r="I2" s="146"/>
+      <c r="J2" s="146"/>
+      <c r="K2" s="147"/>
+    </row>
+    <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="32"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="68"/>
-    </row>
-    <row r="4" spans="1:22" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D3" s="146"/>
+      <c r="E3" s="146"/>
+      <c r="F3" s="146"/>
+      <c r="G3" s="146"/>
+      <c r="H3" s="146"/>
+      <c r="I3" s="146"/>
+      <c r="J3" s="146"/>
+      <c r="K3" s="147"/>
+    </row>
+    <row r="4" spans="1:11" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
       <c r="B4" s="25"/>
       <c r="C4" s="25"/>
@@ -2706,238 +2662,173 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="32"/>
       <c r="K5" s="49"/>
     </row>
-    <row r="6" spans="1:22" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="79" t="s">
+    <row r="6" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="158" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="80"/>
-      <c r="C6" s="80"/>
-      <c r="D6" s="80"/>
-      <c r="E6" s="80"/>
-      <c r="F6" s="80"/>
-      <c r="G6" s="80"/>
-      <c r="H6" s="80"/>
-      <c r="I6" s="79" t="s">
+      <c r="B6" s="159"/>
+      <c r="C6" s="159"/>
+      <c r="D6" s="159"/>
+      <c r="E6" s="159"/>
+      <c r="F6" s="159"/>
+      <c r="G6" s="159"/>
+      <c r="H6" s="159"/>
+      <c r="I6" s="158" t="s">
         <v>1</v>
       </c>
-      <c r="J6" s="80"/>
-      <c r="K6" s="81"/>
-    </row>
-    <row r="7" spans="1:22" s="7" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="85" t="s">
+      <c r="J6" s="159"/>
+      <c r="K6" s="160"/>
+    </row>
+    <row r="7" spans="1:11" s="7" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="164" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="86"/>
-      <c r="C7" s="86"/>
-      <c r="D7" s="86"/>
-      <c r="E7" s="86"/>
-      <c r="F7" s="86"/>
-      <c r="G7" s="86"/>
-      <c r="H7" s="87"/>
-      <c r="I7" s="82" t="s">
+      <c r="B7" s="165"/>
+      <c r="C7" s="165"/>
+      <c r="D7" s="165"/>
+      <c r="E7" s="165"/>
+      <c r="F7" s="165"/>
+      <c r="G7" s="165"/>
+      <c r="H7" s="166"/>
+      <c r="I7" s="161" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="83"/>
-      <c r="K7" s="84"/>
-    </row>
-    <row r="8" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="88" t="s">
-        <v>102</v>
-      </c>
-      <c r="B8" s="89"/>
-      <c r="C8" s="89"/>
-      <c r="D8" s="89"/>
-      <c r="E8" s="89"/>
-      <c r="F8" s="89"/>
-      <c r="G8" s="89"/>
-      <c r="H8" s="90"/>
+      <c r="J7" s="162"/>
+      <c r="K7" s="163"/>
+    </row>
+    <row r="8" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="167" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="168"/>
+      <c r="C8" s="168"/>
+      <c r="D8" s="168"/>
+      <c r="E8" s="168"/>
+      <c r="F8" s="168"/>
+      <c r="G8" s="168"/>
+      <c r="H8" s="169"/>
       <c r="I8" s="8"/>
       <c r="J8" s="9"/>
       <c r="K8" s="10"/>
-      <c r="M8" s="58" t="str">
-        <f>'Cadastro Parte 2'!A41</f>
-        <v>CLIENTE NOVO</v>
-      </c>
-      <c r="N8" s="59"/>
-      <c r="O8" s="59"/>
-      <c r="P8" s="59"/>
-      <c r="Q8" s="59"/>
-      <c r="R8" s="59"/>
-      <c r="S8" s="59"/>
-      <c r="T8" s="59"/>
-      <c r="U8" s="59"/>
-      <c r="V8" s="60"/>
-    </row>
-    <row r="9" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="91" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="92"/>
-      <c r="C9" s="92"/>
-      <c r="D9" s="92"/>
-      <c r="E9" s="92"/>
-      <c r="F9" s="92"/>
-      <c r="G9" s="92"/>
-      <c r="H9" s="93"/>
+    </row>
+    <row r="9" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="170" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="171"/>
+      <c r="C9" s="171"/>
+      <c r="D9" s="171"/>
+      <c r="E9" s="171"/>
+      <c r="F9" s="171"/>
+      <c r="G9" s="171"/>
+      <c r="H9" s="172"/>
       <c r="I9" s="8" t="s">
         <v>4</v>
       </c>
       <c r="J9" s="9"/>
       <c r="K9" s="10"/>
-      <c r="M9" s="61" t="str">
-        <f>'Cadastro Parte 2'!A42</f>
-        <v>Lojista = (Produto para Comercializar / Revender)</v>
-      </c>
-      <c r="N9" s="62"/>
-      <c r="O9" s="62"/>
-      <c r="P9" s="62"/>
-      <c r="Q9" s="62"/>
-      <c r="R9" s="62"/>
-      <c r="S9" s="62"/>
-      <c r="T9" s="62"/>
-      <c r="U9" s="62"/>
-      <c r="V9" s="63"/>
-    </row>
-    <row r="10" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="91" t="s">
-        <v>92</v>
-      </c>
-      <c r="B10" s="92"/>
-      <c r="C10" s="92"/>
-      <c r="D10" s="92"/>
-      <c r="E10" s="92"/>
-      <c r="F10" s="92"/>
-      <c r="G10" s="92"/>
-      <c r="H10" s="93"/>
+    </row>
+    <row r="10" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="170" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" s="171"/>
+      <c r="C10" s="171"/>
+      <c r="D10" s="171"/>
+      <c r="E10" s="171"/>
+      <c r="F10" s="171"/>
+      <c r="G10" s="171"/>
+      <c r="H10" s="172"/>
       <c r="I10" s="11"/>
       <c r="J10" s="12"/>
       <c r="K10" s="13"/>
-      <c r="M10" s="61" t="str">
-        <f>'Cadastro Parte 2'!A43</f>
-        <v>Venda a Prazo</v>
-      </c>
-      <c r="N10" s="62"/>
-      <c r="O10" s="62"/>
-      <c r="P10" s="62"/>
-      <c r="Q10" s="62"/>
-      <c r="R10" s="62"/>
-      <c r="S10" s="62"/>
-      <c r="T10" s="62"/>
-      <c r="U10" s="62"/>
-      <c r="V10" s="63"/>
-    </row>
-    <row r="11" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="94" t="s">
+    </row>
+    <row r="11" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="173" t="s">
+        <v>102</v>
+      </c>
+      <c r="B11" s="174"/>
+      <c r="C11" s="174"/>
+      <c r="D11" s="174"/>
+      <c r="E11" s="148" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11" s="149"/>
+      <c r="G11" s="149"/>
+      <c r="H11" s="149"/>
+      <c r="I11" s="149"/>
+      <c r="J11" s="149"/>
+      <c r="K11" s="150"/>
+    </row>
+    <row r="12" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="173" t="s">
+        <v>103</v>
+      </c>
+      <c r="B12" s="174"/>
+      <c r="C12" s="174"/>
+      <c r="D12" s="174"/>
+      <c r="E12" s="175" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="175"/>
+      <c r="G12" s="175"/>
+      <c r="H12" s="175"/>
+      <c r="I12" s="175"/>
+      <c r="J12" s="175"/>
+      <c r="K12" s="176"/>
+    </row>
+    <row r="13" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="173" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" s="174"/>
+      <c r="C13" s="174"/>
+      <c r="D13" s="174"/>
+      <c r="E13" s="174" t="s">
         <v>104</v>
       </c>
-      <c r="B11" s="95"/>
-      <c r="C11" s="95"/>
-      <c r="D11" s="95"/>
-      <c r="E11" s="69" t="s">
-        <v>99</v>
-      </c>
-      <c r="F11" s="70"/>
-      <c r="G11" s="70"/>
-      <c r="H11" s="70"/>
-      <c r="I11" s="70"/>
-      <c r="J11" s="70"/>
-      <c r="K11" s="71"/>
-      <c r="M11" s="61">
-        <f>'Cadastro Parte 2'!A44</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="62"/>
-      <c r="O11" s="62"/>
-      <c r="P11" s="62"/>
-      <c r="Q11" s="62"/>
-      <c r="R11" s="62"/>
-      <c r="S11" s="62"/>
-      <c r="T11" s="62"/>
-      <c r="U11" s="62"/>
-      <c r="V11" s="63"/>
-    </row>
-    <row r="12" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="94" t="s">
-        <v>105</v>
-      </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="96" t="s">
-        <v>67</v>
-      </c>
-      <c r="F12" s="96"/>
-      <c r="G12" s="96"/>
-      <c r="H12" s="96"/>
-      <c r="I12" s="96"/>
-      <c r="J12" s="96"/>
-      <c r="K12" s="97"/>
-      <c r="M12" s="64">
-        <f>'Cadastro Parte 2'!A45</f>
-        <v>0</v>
-      </c>
-      <c r="N12" s="65"/>
-      <c r="O12" s="65"/>
-      <c r="P12" s="65"/>
-      <c r="Q12" s="65"/>
-      <c r="R12" s="65"/>
-      <c r="S12" s="65"/>
-      <c r="T12" s="65"/>
-      <c r="U12" s="65"/>
-      <c r="V12" s="66"/>
-    </row>
-    <row r="13" spans="1:22" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="94" t="s">
-        <v>91</v>
-      </c>
-      <c r="B13" s="95"/>
-      <c r="C13" s="95"/>
-      <c r="D13" s="95"/>
-      <c r="E13" s="95" t="s">
-        <v>106</v>
-      </c>
-      <c r="F13" s="95"/>
-      <c r="G13" s="95"/>
-      <c r="H13" s="95"/>
-      <c r="I13" s="95"/>
-      <c r="J13" s="95"/>
-      <c r="K13" s="98"/>
-    </row>
-    <row r="14" spans="1:22" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="103" t="s">
+      <c r="F13" s="174"/>
+      <c r="G13" s="174"/>
+      <c r="H13" s="174"/>
+      <c r="I13" s="174"/>
+      <c r="J13" s="174"/>
+      <c r="K13" s="177"/>
+    </row>
+    <row r="14" spans="1:11" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="136" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="104"/>
-      <c r="C14" s="104"/>
-      <c r="D14" s="104"/>
-      <c r="E14" s="104"/>
-      <c r="F14" s="104"/>
-      <c r="G14" s="104"/>
-      <c r="H14" s="104"/>
-      <c r="I14" s="104"/>
-      <c r="J14" s="104"/>
-      <c r="K14" s="105"/>
-    </row>
-    <row r="15" spans="1:22" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="72" t="s">
+      <c r="B14" s="137"/>
+      <c r="C14" s="137"/>
+      <c r="D14" s="137"/>
+      <c r="E14" s="137"/>
+      <c r="F14" s="137"/>
+      <c r="G14" s="137"/>
+      <c r="H14" s="137"/>
+      <c r="I14" s="137"/>
+      <c r="J14" s="137"/>
+      <c r="K14" s="138"/>
+    </row>
+    <row r="15" spans="1:11" s="7" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="151" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="73"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="73"/>
-      <c r="F15" s="73"/>
-      <c r="G15" s="73"/>
-      <c r="H15" s="73"/>
-      <c r="I15" s="73"/>
-      <c r="J15" s="73"/>
-      <c r="K15" s="74"/>
-    </row>
-    <row r="16" spans="1:22" s="7" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="152"/>
+      <c r="C15" s="152"/>
+      <c r="D15" s="152"/>
+      <c r="E15" s="152"/>
+      <c r="F15" s="152"/>
+      <c r="G15" s="152"/>
+      <c r="H15" s="152"/>
+      <c r="I15" s="152"/>
+      <c r="J15" s="152"/>
+      <c r="K15" s="153"/>
+    </row>
+    <row r="16" spans="1:11" s="7" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="35" t="s">
         <v>69</v>
       </c>
@@ -2953,48 +2844,48 @@
       <c r="K16" s="28"/>
     </row>
     <row r="17" spans="1:11" s="7" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="99" t="s">
+      <c r="A17" s="132" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="100"/>
-      <c r="C17" s="75" t="s">
+      <c r="B17" s="133"/>
+      <c r="C17" s="154" t="s">
         <v>70</v>
       </c>
-      <c r="D17" s="76"/>
-      <c r="E17" s="75" t="s">
-        <v>100</v>
-      </c>
-      <c r="F17" s="76"/>
-      <c r="G17" s="75" t="s">
+      <c r="D17" s="155"/>
+      <c r="E17" s="154" t="s">
+        <v>99</v>
+      </c>
+      <c r="F17" s="155"/>
+      <c r="G17" s="154" t="s">
         <v>72</v>
       </c>
-      <c r="H17" s="76"/>
-      <c r="I17" s="75" t="s">
+      <c r="H17" s="155"/>
+      <c r="I17" s="154" t="s">
         <v>74</v>
       </c>
-      <c r="J17" s="77"/>
-      <c r="K17" s="78"/>
+      <c r="J17" s="156"/>
+      <c r="K17" s="157"/>
     </row>
     <row r="18" spans="1:11" s="7" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="106" t="s">
-        <v>107</v>
-      </c>
-      <c r="D18" s="107"/>
-      <c r="E18" s="106" t="s">
+      <c r="A18" s="134"/>
+      <c r="B18" s="135"/>
+      <c r="C18" s="139" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" s="140"/>
+      <c r="E18" s="139" t="s">
         <v>71</v>
       </c>
-      <c r="F18" s="107"/>
-      <c r="G18" s="106" t="s">
+      <c r="F18" s="140"/>
+      <c r="G18" s="139" t="s">
         <v>73</v>
       </c>
-      <c r="H18" s="107"/>
-      <c r="I18" s="106" t="s">
+      <c r="H18" s="140"/>
+      <c r="I18" s="139" t="s">
         <v>75</v>
       </c>
-      <c r="J18" s="117"/>
-      <c r="K18" s="118"/>
+      <c r="J18" s="141"/>
+      <c r="K18" s="142"/>
     </row>
     <row r="19" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="50"/>
@@ -3010,55 +2901,55 @@
       <c r="K19" s="46"/>
     </row>
     <row r="20" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="111" t="s">
+      <c r="A20" s="93" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="112"/>
-      <c r="C20" s="112"/>
-      <c r="D20" s="112"/>
-      <c r="E20" s="112"/>
-      <c r="F20" s="112"/>
-      <c r="G20" s="112"/>
-      <c r="H20" s="112"/>
-      <c r="I20" s="112"/>
-      <c r="J20" s="112"/>
-      <c r="K20" s="113"/>
+      <c r="B20" s="94"/>
+      <c r="C20" s="94"/>
+      <c r="D20" s="94"/>
+      <c r="E20" s="94"/>
+      <c r="F20" s="94"/>
+      <c r="G20" s="94"/>
+      <c r="H20" s="94"/>
+      <c r="I20" s="94"/>
+      <c r="J20" s="94"/>
+      <c r="K20" s="95"/>
     </row>
     <row r="21" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="119" t="s">
-        <v>93</v>
-      </c>
-      <c r="B21" s="120"/>
-      <c r="C21" s="120"/>
-      <c r="D21" s="120"/>
-      <c r="E21" s="120"/>
-      <c r="F21" s="120"/>
-      <c r="G21" s="120"/>
-      <c r="H21" s="121"/>
-      <c r="I21" s="122" t="s">
+      <c r="A21" s="143" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" s="144"/>
+      <c r="C21" s="144"/>
+      <c r="D21" s="144"/>
+      <c r="E21" s="144"/>
+      <c r="F21" s="144"/>
+      <c r="G21" s="144"/>
+      <c r="H21" s="145"/>
+      <c r="I21" s="119" t="s">
+        <v>106</v>
+      </c>
+      <c r="J21" s="120"/>
+      <c r="K21" s="121"/>
+    </row>
+    <row r="22" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="83" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" s="84"/>
+      <c r="C22" s="84"/>
+      <c r="D22" s="84"/>
+      <c r="E22" s="84"/>
+      <c r="F22" s="122" t="s">
         <v>108</v>
       </c>
-      <c r="J21" s="123"/>
-      <c r="K21" s="124"/>
-    </row>
-    <row r="22" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="108" t="s">
-        <v>95</v>
-      </c>
-      <c r="B22" s="109"/>
-      <c r="C22" s="109"/>
-      <c r="D22" s="109"/>
-      <c r="E22" s="109"/>
-      <c r="F22" s="114" t="s">
-        <v>110</v>
-      </c>
-      <c r="G22" s="109"/>
-      <c r="H22" s="115"/>
-      <c r="I22" s="114" t="s">
-        <v>109</v>
-      </c>
-      <c r="J22" s="109"/>
-      <c r="K22" s="116"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="85"/>
+      <c r="I22" s="122" t="s">
+        <v>107</v>
+      </c>
+      <c r="J22" s="84"/>
+      <c r="K22" s="123"/>
     </row>
     <row r="23" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="50"/>
@@ -3074,55 +2965,55 @@
       <c r="K23" s="48"/>
     </row>
     <row r="24" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="111" t="s">
+      <c r="A24" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="112"/>
-      <c r="C24" s="112"/>
-      <c r="D24" s="112"/>
-      <c r="E24" s="112"/>
-      <c r="F24" s="112"/>
-      <c r="G24" s="112"/>
-      <c r="H24" s="112"/>
-      <c r="I24" s="112"/>
-      <c r="J24" s="112"/>
-      <c r="K24" s="113"/>
+      <c r="B24" s="94"/>
+      <c r="C24" s="94"/>
+      <c r="D24" s="94"/>
+      <c r="E24" s="94"/>
+      <c r="F24" s="94"/>
+      <c r="G24" s="94"/>
+      <c r="H24" s="94"/>
+      <c r="I24" s="94"/>
+      <c r="J24" s="94"/>
+      <c r="K24" s="95"/>
     </row>
     <row r="25" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="132" t="s">
+      <c r="A25" s="126" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" s="127"/>
+      <c r="C25" s="127"/>
+      <c r="D25" s="127"/>
+      <c r="E25" s="127"/>
+      <c r="F25" s="127"/>
+      <c r="G25" s="127"/>
+      <c r="H25" s="128"/>
+      <c r="I25" s="119" t="s">
         <v>93</v>
       </c>
-      <c r="B25" s="133"/>
-      <c r="C25" s="133"/>
-      <c r="D25" s="133"/>
-      <c r="E25" s="133"/>
-      <c r="F25" s="133"/>
-      <c r="G25" s="133"/>
-      <c r="H25" s="134"/>
-      <c r="I25" s="122" t="s">
+      <c r="J25" s="120"/>
+      <c r="K25" s="121"/>
+    </row>
+    <row r="26" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="83" t="s">
         <v>94</v>
       </c>
-      <c r="J25" s="123"/>
-      <c r="K25" s="124"/>
-    </row>
-    <row r="26" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="108" t="s">
+      <c r="B26" s="84"/>
+      <c r="C26" s="84"/>
+      <c r="D26" s="84"/>
+      <c r="E26" s="84"/>
+      <c r="F26" s="122" t="s">
         <v>95</v>
       </c>
-      <c r="B26" s="109"/>
-      <c r="C26" s="109"/>
-      <c r="D26" s="109"/>
-      <c r="E26" s="109"/>
-      <c r="F26" s="114" t="s">
+      <c r="G26" s="84"/>
+      <c r="H26" s="85"/>
+      <c r="I26" s="122" t="s">
         <v>96</v>
       </c>
-      <c r="G26" s="109"/>
-      <c r="H26" s="115"/>
-      <c r="I26" s="114" t="s">
-        <v>97</v>
-      </c>
-      <c r="J26" s="109"/>
-      <c r="K26" s="116"/>
+      <c r="J26" s="84"/>
+      <c r="K26" s="123"/>
     </row>
     <row r="27" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="50"/>
@@ -3138,53 +3029,53 @@
       <c r="K27" s="48"/>
     </row>
     <row r="28" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="111" t="s">
+      <c r="A28" s="93" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="112"/>
-      <c r="C28" s="112"/>
-      <c r="D28" s="112"/>
-      <c r="E28" s="112"/>
-      <c r="F28" s="112"/>
-      <c r="G28" s="112"/>
-      <c r="H28" s="112"/>
-      <c r="I28" s="112"/>
-      <c r="J28" s="112"/>
-      <c r="K28" s="113"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="94"/>
+      <c r="F28" s="94"/>
+      <c r="G28" s="94"/>
+      <c r="H28" s="94"/>
+      <c r="I28" s="94"/>
+      <c r="J28" s="94"/>
+      <c r="K28" s="95"/>
     </row>
     <row r="29" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="130" t="s">
+      <c r="A29" s="124" t="s">
+        <v>109</v>
+      </c>
+      <c r="B29" s="125"/>
+      <c r="C29" s="125"/>
+      <c r="D29" s="125"/>
+      <c r="E29" s="125"/>
+      <c r="F29" s="119" t="s">
         <v>111</v>
       </c>
-      <c r="B29" s="131"/>
-      <c r="C29" s="131"/>
-      <c r="D29" s="131"/>
-      <c r="E29" s="131"/>
-      <c r="F29" s="122" t="s">
-        <v>113</v>
-      </c>
-      <c r="G29" s="123"/>
-      <c r="H29" s="123"/>
-      <c r="I29" s="123"/>
-      <c r="J29" s="123"/>
-      <c r="K29" s="124"/>
+      <c r="G29" s="120"/>
+      <c r="H29" s="120"/>
+      <c r="I29" s="120"/>
+      <c r="J29" s="120"/>
+      <c r="K29" s="121"/>
     </row>
     <row r="30" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="139" t="s">
+      <c r="A30" s="72" t="s">
+        <v>110</v>
+      </c>
+      <c r="B30" s="73"/>
+      <c r="C30" s="73"/>
+      <c r="D30" s="73"/>
+      <c r="E30" s="73"/>
+      <c r="F30" s="129" t="s">
         <v>112</v>
       </c>
-      <c r="B30" s="140"/>
-      <c r="C30" s="140"/>
-      <c r="D30" s="140"/>
-      <c r="E30" s="140"/>
-      <c r="F30" s="141" t="s">
-        <v>114</v>
-      </c>
-      <c r="G30" s="142"/>
-      <c r="H30" s="142"/>
-      <c r="I30" s="142"/>
-      <c r="J30" s="142"/>
-      <c r="K30" s="143"/>
+      <c r="G30" s="130"/>
+      <c r="H30" s="130"/>
+      <c r="I30" s="130"/>
+      <c r="J30" s="130"/>
+      <c r="K30" s="131"/>
     </row>
     <row r="31" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="50"/>
@@ -3200,83 +3091,83 @@
       <c r="K31" s="48"/>
     </row>
     <row r="32" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="111" t="s">
+      <c r="A32" s="93" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="112"/>
-      <c r="C32" s="112"/>
-      <c r="D32" s="112"/>
-      <c r="E32" s="112"/>
-      <c r="F32" s="112"/>
-      <c r="G32" s="112"/>
-      <c r="H32" s="112"/>
-      <c r="I32" s="112"/>
-      <c r="J32" s="112"/>
-      <c r="K32" s="113"/>
+      <c r="B32" s="94"/>
+      <c r="C32" s="94"/>
+      <c r="D32" s="94"/>
+      <c r="E32" s="94"/>
+      <c r="F32" s="94"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="94"/>
+      <c r="I32" s="94"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="95"/>
     </row>
     <row r="33" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="128" t="s">
+      <c r="A33" s="117" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="129"/>
-      <c r="C33" s="110" t="s">
+      <c r="B33" s="118"/>
+      <c r="C33" s="97" t="s">
         <v>12</v>
       </c>
-      <c r="D33" s="110"/>
-      <c r="E33" s="110" t="s">
+      <c r="D33" s="97"/>
+      <c r="E33" s="97" t="s">
         <v>13</v>
       </c>
-      <c r="F33" s="110"/>
+      <c r="F33" s="97"/>
       <c r="G33" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="H33" s="110" t="s">
+      <c r="H33" s="97" t="s">
         <v>14</v>
       </c>
-      <c r="I33" s="110"/>
-      <c r="J33" s="110" t="s">
+      <c r="I33" s="97"/>
+      <c r="J33" s="97" t="s">
         <v>15</v>
       </c>
-      <c r="K33" s="126"/>
+      <c r="K33" s="98"/>
     </row>
     <row r="34" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="137"/>
-      <c r="B34" s="138"/>
-      <c r="C34" s="135"/>
-      <c r="D34" s="136"/>
-      <c r="E34" s="135"/>
-      <c r="F34" s="136"/>
+      <c r="A34" s="77"/>
+      <c r="B34" s="78"/>
+      <c r="C34" s="87"/>
+      <c r="D34" s="88"/>
+      <c r="E34" s="87"/>
+      <c r="F34" s="88"/>
       <c r="G34" s="55"/>
-      <c r="H34" s="125"/>
-      <c r="I34" s="125"/>
-      <c r="J34" s="125"/>
-      <c r="K34" s="127"/>
+      <c r="H34" s="70"/>
+      <c r="I34" s="70"/>
+      <c r="J34" s="70"/>
+      <c r="K34" s="71"/>
     </row>
     <row r="35" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="137"/>
-      <c r="B35" s="138"/>
-      <c r="C35" s="125"/>
-      <c r="D35" s="125"/>
-      <c r="E35" s="125"/>
-      <c r="F35" s="125"/>
+      <c r="A35" s="77"/>
+      <c r="B35" s="78"/>
+      <c r="C35" s="70"/>
+      <c r="D35" s="70"/>
+      <c r="E35" s="70"/>
+      <c r="F35" s="70"/>
       <c r="G35" s="55"/>
-      <c r="H35" s="125"/>
-      <c r="I35" s="125"/>
-      <c r="J35" s="125"/>
-      <c r="K35" s="127"/>
+      <c r="H35" s="70"/>
+      <c r="I35" s="70"/>
+      <c r="J35" s="70"/>
+      <c r="K35" s="71"/>
     </row>
     <row r="36" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="139"/>
-      <c r="B36" s="140"/>
-      <c r="C36" s="145"/>
-      <c r="D36" s="145"/>
-      <c r="E36" s="145"/>
-      <c r="F36" s="145"/>
+      <c r="A36" s="72"/>
+      <c r="B36" s="73"/>
+      <c r="C36" s="75"/>
+      <c r="D36" s="75"/>
+      <c r="E36" s="75"/>
+      <c r="F36" s="75"/>
       <c r="G36" s="56"/>
-      <c r="H36" s="145"/>
-      <c r="I36" s="145"/>
-      <c r="J36" s="145"/>
-      <c r="K36" s="146"/>
+      <c r="H36" s="75"/>
+      <c r="I36" s="75"/>
+      <c r="J36" s="75"/>
+      <c r="K36" s="76"/>
     </row>
     <row r="37" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="50"/>
@@ -3292,79 +3183,79 @@
       <c r="K37" s="51"/>
     </row>
     <row r="38" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="111" t="s">
+      <c r="A38" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="B38" s="112"/>
-      <c r="C38" s="112"/>
-      <c r="D38" s="112"/>
-      <c r="E38" s="112"/>
-      <c r="F38" s="112"/>
-      <c r="G38" s="112"/>
-      <c r="H38" s="112"/>
-      <c r="I38" s="112"/>
-      <c r="J38" s="112"/>
-      <c r="K38" s="113"/>
+      <c r="B38" s="94"/>
+      <c r="C38" s="94"/>
+      <c r="D38" s="94"/>
+      <c r="E38" s="94"/>
+      <c r="F38" s="94"/>
+      <c r="G38" s="94"/>
+      <c r="H38" s="94"/>
+      <c r="I38" s="94"/>
+      <c r="J38" s="94"/>
+      <c r="K38" s="95"/>
     </row>
     <row r="39" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="144" t="s">
+      <c r="A39" s="96" t="s">
         <v>19</v>
       </c>
-      <c r="B39" s="110"/>
-      <c r="C39" s="110"/>
-      <c r="D39" s="110"/>
-      <c r="E39" s="110" t="s">
+      <c r="B39" s="97"/>
+      <c r="C39" s="97"/>
+      <c r="D39" s="97"/>
+      <c r="E39" s="97" t="s">
         <v>20</v>
       </c>
-      <c r="F39" s="110"/>
-      <c r="G39" s="110" t="s">
+      <c r="F39" s="97"/>
+      <c r="G39" s="97" t="s">
         <v>14</v>
       </c>
-      <c r="H39" s="110"/>
-      <c r="I39" s="110" t="s">
+      <c r="H39" s="97"/>
+      <c r="I39" s="97" t="s">
         <v>15</v>
       </c>
-      <c r="J39" s="110"/>
-      <c r="K39" s="126"/>
+      <c r="J39" s="97"/>
+      <c r="K39" s="98"/>
     </row>
     <row r="40" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="154"/>
-      <c r="B40" s="155"/>
-      <c r="C40" s="155"/>
-      <c r="D40" s="156"/>
-      <c r="E40" s="135"/>
-      <c r="F40" s="136"/>
-      <c r="G40" s="135"/>
-      <c r="H40" s="136"/>
-      <c r="I40" s="135"/>
-      <c r="J40" s="157"/>
-      <c r="K40" s="158"/>
+      <c r="A40" s="113"/>
+      <c r="B40" s="114"/>
+      <c r="C40" s="114"/>
+      <c r="D40" s="115"/>
+      <c r="E40" s="87"/>
+      <c r="F40" s="88"/>
+      <c r="G40" s="87"/>
+      <c r="H40" s="88"/>
+      <c r="I40" s="87"/>
+      <c r="J40" s="116"/>
+      <c r="K40" s="91"/>
     </row>
     <row r="41" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="154"/>
-      <c r="B41" s="155"/>
-      <c r="C41" s="155"/>
-      <c r="D41" s="156"/>
-      <c r="E41" s="135"/>
-      <c r="F41" s="136"/>
-      <c r="G41" s="135"/>
-      <c r="H41" s="136"/>
-      <c r="I41" s="135"/>
-      <c r="J41" s="157"/>
-      <c r="K41" s="158"/>
+      <c r="A41" s="113"/>
+      <c r="B41" s="114"/>
+      <c r="C41" s="114"/>
+      <c r="D41" s="115"/>
+      <c r="E41" s="87"/>
+      <c r="F41" s="88"/>
+      <c r="G41" s="87"/>
+      <c r="H41" s="88"/>
+      <c r="I41" s="87"/>
+      <c r="J41" s="116"/>
+      <c r="K41" s="91"/>
     </row>
     <row r="42" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="147"/>
-      <c r="B42" s="148"/>
-      <c r="C42" s="148"/>
-      <c r="D42" s="149"/>
-      <c r="E42" s="150"/>
-      <c r="F42" s="151"/>
-      <c r="G42" s="150"/>
-      <c r="H42" s="151"/>
-      <c r="I42" s="150"/>
-      <c r="J42" s="152"/>
-      <c r="K42" s="153"/>
+      <c r="A42" s="106"/>
+      <c r="B42" s="107"/>
+      <c r="C42" s="107"/>
+      <c r="D42" s="108"/>
+      <c r="E42" s="109"/>
+      <c r="F42" s="110"/>
+      <c r="G42" s="109"/>
+      <c r="H42" s="110"/>
+      <c r="I42" s="109"/>
+      <c r="J42" s="111"/>
+      <c r="K42" s="112"/>
     </row>
     <row r="43" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="50"/>
@@ -3380,68 +3271,68 @@
       <c r="K43" s="51"/>
     </row>
     <row r="44" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="111" t="s">
+      <c r="A44" s="93" t="s">
         <v>21</v>
       </c>
-      <c r="B44" s="112"/>
-      <c r="C44" s="112"/>
-      <c r="D44" s="112"/>
-      <c r="E44" s="112"/>
-      <c r="F44" s="112"/>
-      <c r="G44" s="112"/>
-      <c r="H44" s="112"/>
-      <c r="I44" s="112"/>
-      <c r="J44" s="112"/>
-      <c r="K44" s="113"/>
+      <c r="B44" s="94"/>
+      <c r="C44" s="94"/>
+      <c r="D44" s="94"/>
+      <c r="E44" s="94"/>
+      <c r="F44" s="94"/>
+      <c r="G44" s="94"/>
+      <c r="H44" s="94"/>
+      <c r="I44" s="94"/>
+      <c r="J44" s="94"/>
+      <c r="K44" s="95"/>
     </row>
     <row r="45" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="144" t="s">
+      <c r="A45" s="96" t="s">
         <v>22</v>
       </c>
-      <c r="B45" s="110"/>
-      <c r="C45" s="110" t="s">
+      <c r="B45" s="97"/>
+      <c r="C45" s="97" t="s">
         <v>23</v>
       </c>
-      <c r="D45" s="110"/>
-      <c r="E45" s="110"/>
-      <c r="F45" s="110" t="s">
+      <c r="D45" s="97"/>
+      <c r="E45" s="97"/>
+      <c r="F45" s="97" t="s">
         <v>24</v>
       </c>
-      <c r="G45" s="110"/>
-      <c r="H45" s="110" t="s">
+      <c r="G45" s="97"/>
+      <c r="H45" s="97" t="s">
         <v>35</v>
       </c>
-      <c r="I45" s="110"/>
-      <c r="J45" s="110" t="s">
+      <c r="I45" s="97"/>
+      <c r="J45" s="97" t="s">
         <v>26</v>
       </c>
-      <c r="K45" s="126"/>
+      <c r="K45" s="98"/>
     </row>
     <row r="46" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="160"/>
-      <c r="B46" s="161"/>
-      <c r="C46" s="125"/>
-      <c r="D46" s="125"/>
-      <c r="E46" s="125"/>
-      <c r="F46" s="125"/>
-      <c r="G46" s="125"/>
-      <c r="H46" s="162"/>
-      <c r="I46" s="162"/>
-      <c r="J46" s="125"/>
-      <c r="K46" s="127"/>
+      <c r="A46" s="80"/>
+      <c r="B46" s="82"/>
+      <c r="C46" s="70"/>
+      <c r="D46" s="70"/>
+      <c r="E46" s="70"/>
+      <c r="F46" s="70"/>
+      <c r="G46" s="70"/>
+      <c r="H46" s="105"/>
+      <c r="I46" s="105"/>
+      <c r="J46" s="70"/>
+      <c r="K46" s="71"/>
     </row>
     <row r="47" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="108"/>
-      <c r="B47" s="115"/>
-      <c r="C47" s="145"/>
-      <c r="D47" s="145"/>
-      <c r="E47" s="145"/>
-      <c r="F47" s="145"/>
-      <c r="G47" s="145"/>
-      <c r="H47" s="159"/>
-      <c r="I47" s="159"/>
-      <c r="J47" s="145"/>
-      <c r="K47" s="146"/>
+      <c r="A47" s="83"/>
+      <c r="B47" s="85"/>
+      <c r="C47" s="75"/>
+      <c r="D47" s="75"/>
+      <c r="E47" s="75"/>
+      <c r="F47" s="75"/>
+      <c r="G47" s="75"/>
+      <c r="H47" s="104"/>
+      <c r="I47" s="104"/>
+      <c r="J47" s="75"/>
+      <c r="K47" s="76"/>
     </row>
     <row r="48" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="50"/>
@@ -3457,79 +3348,79 @@
       <c r="K48" s="51"/>
     </row>
     <row r="49" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="111" t="s">
+      <c r="A49" s="93" t="s">
         <v>27</v>
       </c>
-      <c r="B49" s="112"/>
-      <c r="C49" s="112"/>
-      <c r="D49" s="112"/>
-      <c r="E49" s="112"/>
-      <c r="F49" s="112"/>
-      <c r="G49" s="112"/>
-      <c r="H49" s="112"/>
-      <c r="I49" s="112"/>
-      <c r="J49" s="112"/>
-      <c r="K49" s="113"/>
+      <c r="B49" s="94"/>
+      <c r="C49" s="94"/>
+      <c r="D49" s="94"/>
+      <c r="E49" s="94"/>
+      <c r="F49" s="94"/>
+      <c r="G49" s="94"/>
+      <c r="H49" s="94"/>
+      <c r="I49" s="94"/>
+      <c r="J49" s="94"/>
+      <c r="K49" s="95"/>
     </row>
     <row r="50" spans="1:11" s="7" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="163" t="s">
+      <c r="A50" s="99" t="s">
         <v>28</v>
       </c>
-      <c r="B50" s="164"/>
-      <c r="C50" s="164"/>
-      <c r="D50" s="164"/>
-      <c r="E50" s="164"/>
-      <c r="F50" s="164" t="s">
+      <c r="B50" s="100"/>
+      <c r="C50" s="100"/>
+      <c r="D50" s="100"/>
+      <c r="E50" s="100"/>
+      <c r="F50" s="100" t="s">
         <v>29</v>
       </c>
-      <c r="G50" s="164"/>
-      <c r="H50" s="166" t="s">
+      <c r="G50" s="100"/>
+      <c r="H50" s="101" t="s">
         <v>76</v>
       </c>
-      <c r="I50" s="167"/>
-      <c r="J50" s="166" t="s">
+      <c r="I50" s="102"/>
+      <c r="J50" s="101" t="s">
         <v>77</v>
       </c>
-      <c r="K50" s="168"/>
+      <c r="K50" s="103"/>
     </row>
     <row r="51" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="160"/>
-      <c r="B51" s="165"/>
-      <c r="C51" s="165"/>
-      <c r="D51" s="165"/>
-      <c r="E51" s="161"/>
-      <c r="F51" s="125"/>
-      <c r="G51" s="125"/>
-      <c r="H51" s="135"/>
-      <c r="I51" s="136"/>
-      <c r="J51" s="135"/>
-      <c r="K51" s="158"/>
+      <c r="A51" s="80"/>
+      <c r="B51" s="81"/>
+      <c r="C51" s="81"/>
+      <c r="D51" s="81"/>
+      <c r="E51" s="82"/>
+      <c r="F51" s="70"/>
+      <c r="G51" s="70"/>
+      <c r="H51" s="87"/>
+      <c r="I51" s="88"/>
+      <c r="J51" s="87"/>
+      <c r="K51" s="91"/>
     </row>
     <row r="52" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="160"/>
-      <c r="B52" s="165"/>
-      <c r="C52" s="165"/>
-      <c r="D52" s="165"/>
-      <c r="E52" s="161"/>
-      <c r="F52" s="125"/>
-      <c r="G52" s="125"/>
-      <c r="H52" s="135"/>
-      <c r="I52" s="136"/>
-      <c r="J52" s="135"/>
-      <c r="K52" s="158"/>
+      <c r="A52" s="80"/>
+      <c r="B52" s="81"/>
+      <c r="C52" s="81"/>
+      <c r="D52" s="81"/>
+      <c r="E52" s="82"/>
+      <c r="F52" s="70"/>
+      <c r="G52" s="70"/>
+      <c r="H52" s="87"/>
+      <c r="I52" s="88"/>
+      <c r="J52" s="87"/>
+      <c r="K52" s="91"/>
     </row>
     <row r="53" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="108"/>
-      <c r="B53" s="109"/>
-      <c r="C53" s="109"/>
-      <c r="D53" s="109"/>
-      <c r="E53" s="115"/>
-      <c r="F53" s="145"/>
-      <c r="G53" s="145"/>
-      <c r="H53" s="170"/>
-      <c r="I53" s="171"/>
-      <c r="J53" s="170"/>
-      <c r="K53" s="172"/>
+      <c r="A53" s="83"/>
+      <c r="B53" s="84"/>
+      <c r="C53" s="84"/>
+      <c r="D53" s="84"/>
+      <c r="E53" s="85"/>
+      <c r="F53" s="75"/>
+      <c r="G53" s="75"/>
+      <c r="H53" s="89"/>
+      <c r="I53" s="90"/>
+      <c r="J53" s="89"/>
+      <c r="K53" s="92"/>
     </row>
     <row r="54" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="52"/>
@@ -3545,109 +3436,109 @@
       <c r="K54" s="51"/>
     </row>
     <row r="55" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="111" t="s">
+      <c r="A55" s="93" t="s">
         <v>53</v>
       </c>
-      <c r="B55" s="112"/>
-      <c r="C55" s="112"/>
-      <c r="D55" s="112"/>
-      <c r="E55" s="112"/>
-      <c r="F55" s="112"/>
-      <c r="G55" s="112"/>
-      <c r="H55" s="112"/>
-      <c r="I55" s="112"/>
-      <c r="J55" s="112"/>
-      <c r="K55" s="113"/>
+      <c r="B55" s="94"/>
+      <c r="C55" s="94"/>
+      <c r="D55" s="94"/>
+      <c r="E55" s="94"/>
+      <c r="F55" s="94"/>
+      <c r="G55" s="94"/>
+      <c r="H55" s="94"/>
+      <c r="I55" s="94"/>
+      <c r="J55" s="94"/>
+      <c r="K55" s="95"/>
     </row>
     <row r="56" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="144" t="s">
+      <c r="A56" s="96" t="s">
         <v>30</v>
       </c>
-      <c r="B56" s="110"/>
-      <c r="C56" s="110"/>
-      <c r="D56" s="110"/>
-      <c r="E56" s="110" t="s">
+      <c r="B56" s="97"/>
+      <c r="C56" s="97"/>
+      <c r="D56" s="97"/>
+      <c r="E56" s="97" t="s">
         <v>31</v>
       </c>
-      <c r="F56" s="110"/>
-      <c r="G56" s="110" t="s">
+      <c r="F56" s="97"/>
+      <c r="G56" s="97" t="s">
         <v>25</v>
       </c>
-      <c r="H56" s="110"/>
-      <c r="I56" s="110" t="s">
+      <c r="H56" s="97"/>
+      <c r="I56" s="97" t="s">
         <v>32</v>
       </c>
-      <c r="J56" s="110"/>
-      <c r="K56" s="126"/>
+      <c r="J56" s="97"/>
+      <c r="K56" s="98"/>
     </row>
     <row r="57" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="137"/>
-      <c r="B57" s="138"/>
-      <c r="C57" s="138"/>
-      <c r="D57" s="138"/>
-      <c r="E57" s="125"/>
-      <c r="F57" s="125"/>
-      <c r="G57" s="169"/>
-      <c r="H57" s="169"/>
-      <c r="I57" s="125"/>
-      <c r="J57" s="125"/>
-      <c r="K57" s="127"/>
+      <c r="A57" s="77"/>
+      <c r="B57" s="78"/>
+      <c r="C57" s="78"/>
+      <c r="D57" s="78"/>
+      <c r="E57" s="70"/>
+      <c r="F57" s="70"/>
+      <c r="G57" s="86"/>
+      <c r="H57" s="86"/>
+      <c r="I57" s="70"/>
+      <c r="J57" s="70"/>
+      <c r="K57" s="71"/>
     </row>
     <row r="58" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="137"/>
-      <c r="B58" s="138"/>
-      <c r="C58" s="138"/>
-      <c r="D58" s="138"/>
-      <c r="E58" s="186"/>
-      <c r="F58" s="186"/>
-      <c r="G58" s="184"/>
-      <c r="H58" s="184"/>
-      <c r="I58" s="125"/>
-      <c r="J58" s="125"/>
-      <c r="K58" s="127"/>
+      <c r="A58" s="77"/>
+      <c r="B58" s="78"/>
+      <c r="C58" s="78"/>
+      <c r="D58" s="78"/>
+      <c r="E58" s="79"/>
+      <c r="F58" s="79"/>
+      <c r="G58" s="69"/>
+      <c r="H58" s="69"/>
+      <c r="I58" s="70"/>
+      <c r="J58" s="70"/>
+      <c r="K58" s="71"/>
     </row>
     <row r="59" spans="1:11" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="139"/>
-      <c r="B59" s="140"/>
-      <c r="C59" s="140"/>
-      <c r="D59" s="140"/>
-      <c r="E59" s="140"/>
-      <c r="F59" s="140"/>
-      <c r="G59" s="185"/>
-      <c r="H59" s="185"/>
-      <c r="I59" s="145"/>
-      <c r="J59" s="145"/>
-      <c r="K59" s="146"/>
+      <c r="A59" s="72"/>
+      <c r="B59" s="73"/>
+      <c r="C59" s="73"/>
+      <c r="D59" s="73"/>
+      <c r="E59" s="73"/>
+      <c r="F59" s="73"/>
+      <c r="G59" s="74"/>
+      <c r="H59" s="74"/>
+      <c r="I59" s="75"/>
+      <c r="J59" s="75"/>
+      <c r="K59" s="76"/>
     </row>
     <row r="60" spans="1:11" s="1" customFormat="1" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="173" t="s">
+      <c r="A60" s="58" t="s">
         <v>82</v>
       </c>
-      <c r="B60" s="174"/>
-      <c r="C60" s="174"/>
-      <c r="D60" s="174"/>
-      <c r="E60" s="174"/>
-      <c r="F60" s="174"/>
-      <c r="G60" s="174"/>
-      <c r="H60" s="174"/>
-      <c r="I60" s="175"/>
-      <c r="J60" s="175"/>
-      <c r="K60" s="176"/>
+      <c r="B60" s="59"/>
+      <c r="C60" s="59"/>
+      <c r="D60" s="59"/>
+      <c r="E60" s="59"/>
+      <c r="F60" s="59"/>
+      <c r="G60" s="59"/>
+      <c r="H60" s="59"/>
+      <c r="I60" s="60"/>
+      <c r="J60" s="60"/>
+      <c r="K60" s="61"/>
     </row>
     <row r="61" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="180" t="s">
+      <c r="A61" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="B61" s="181"/>
-      <c r="C61" s="182"/>
-      <c r="D61" s="182"/>
-      <c r="E61" s="182"/>
-      <c r="F61" s="182"/>
-      <c r="G61" s="182"/>
-      <c r="H61" s="182"/>
-      <c r="I61" s="182"/>
-      <c r="J61" s="182"/>
-      <c r="K61" s="183"/>
+      <c r="B61" s="66"/>
+      <c r="C61" s="67"/>
+      <c r="D61" s="67"/>
+      <c r="E61" s="67"/>
+      <c r="F61" s="67"/>
+      <c r="G61" s="67"/>
+      <c r="H61" s="67"/>
+      <c r="I61" s="67"/>
+      <c r="J61" s="67"/>
+      <c r="K61" s="68"/>
     </row>
     <row r="62" spans="1:11" s="1" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="22"/>
@@ -3663,20 +3554,20 @@
       <c r="K62" s="23"/>
     </row>
     <row r="63" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="177" t="s">
+      <c r="A63" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="B63" s="178"/>
-      <c r="C63" s="178"/>
-      <c r="D63" s="178"/>
-      <c r="E63" s="178"/>
-      <c r="G63" s="178" t="s">
+      <c r="B63" s="63"/>
+      <c r="C63" s="63"/>
+      <c r="D63" s="63"/>
+      <c r="E63" s="63"/>
+      <c r="G63" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="H63" s="178"/>
-      <c r="I63" s="178"/>
-      <c r="J63" s="178"/>
-      <c r="K63" s="179"/>
+      <c r="H63" s="63"/>
+      <c r="I63" s="63"/>
+      <c r="J63" s="63"/>
+      <c r="K63" s="64"/>
     </row>
     <row r="64" spans="1:11" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="24"/>
@@ -3692,85 +3583,41 @@
       <c r="K64" s="26"/>
     </row>
   </sheetData>
-  <mergeCells count="141">
-    <mergeCell ref="A60:H60"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="A63:E63"/>
-    <mergeCell ref="G63:K63"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="C61:K61"/>
-    <mergeCell ref="G58:H58"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="G59:H59"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="G57:H57"/>
-    <mergeCell ref="H52:I52"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="J52:K52"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="A55:K55"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="G56:H56"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="A49:K49"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="H51:I51"/>
-    <mergeCell ref="J51:K51"/>
-    <mergeCell ref="H50:I50"/>
-    <mergeCell ref="J50:K50"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="J46:K46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="J47:K47"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="A38:K38"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="H36:I36"/>
+  <mergeCells count="136">
+    <mergeCell ref="D2:K3"/>
+    <mergeCell ref="E11:K11"/>
+    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="E12:K12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="E13:K13"/>
+    <mergeCell ref="A17:B18"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="I21:K21"/>
     <mergeCell ref="H34:I34"/>
     <mergeCell ref="J33:K33"/>
     <mergeCell ref="J34:K34"/>
@@ -3795,45 +3642,84 @@
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="F30:K30"/>
     <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A17:B18"/>
-    <mergeCell ref="A14:K14"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="A24:K24"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="A20:K20"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="M8:V8"/>
-    <mergeCell ref="M9:V9"/>
-    <mergeCell ref="M10:V10"/>
-    <mergeCell ref="M11:V11"/>
-    <mergeCell ref="M12:V12"/>
-    <mergeCell ref="D2:K3"/>
-    <mergeCell ref="E11:K11"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="E12:K12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="E13:K13"/>
+    <mergeCell ref="A38:K38"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="J46:K46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="J47:K47"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="A49:K49"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="J51:K51"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="J50:K50"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="J52:K52"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="A55:K55"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="G56:H56"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="G63:K63"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="C61:K61"/>
+    <mergeCell ref="G58:H58"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="G59:H59"/>
+    <mergeCell ref="I59:K59"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="E58:F58"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -3875,41 +3761,41 @@
     </row>
     <row r="2" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="32"/>
-      <c r="D2" s="67" t="s">
+      <c r="D2" s="146" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="68"/>
+      <c r="E2" s="146"/>
+      <c r="F2" s="146"/>
+      <c r="G2" s="146"/>
+      <c r="H2" s="146"/>
+      <c r="I2" s="146"/>
+      <c r="J2" s="146"/>
+      <c r="K2" s="147"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="32"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="68"/>
+      <c r="D3" s="146"/>
+      <c r="E3" s="146"/>
+      <c r="F3" s="146"/>
+      <c r="G3" s="146"/>
+      <c r="H3" s="146"/>
+      <c r="I3" s="146"/>
+      <c r="J3" s="146"/>
+      <c r="K3" s="147"/>
     </row>
     <row r="4" spans="1:11" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
       <c r="B4" s="25"/>
       <c r="C4" s="25"/>
-      <c r="D4" s="238" t="s">
+      <c r="D4" s="178" t="s">
         <v>84</v>
       </c>
-      <c r="E4" s="238"/>
-      <c r="F4" s="238"/>
-      <c r="G4" s="238"/>
-      <c r="H4" s="238"/>
-      <c r="I4" s="238"/>
-      <c r="J4" s="238"/>
+      <c r="E4" s="178"/>
+      <c r="F4" s="178"/>
+      <c r="G4" s="178"/>
+      <c r="H4" s="178"/>
+      <c r="I4" s="178"/>
+      <c r="J4" s="178"/>
       <c r="K4" s="34" t="s">
         <v>83</v>
       </c>
@@ -3926,53 +3812,53 @@
       <c r="K5" s="23"/>
     </row>
     <row r="6" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="243" t="s">
+      <c r="A6" s="186" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="244"/>
-      <c r="C6" s="244"/>
-      <c r="D6" s="244"/>
-      <c r="E6" s="244"/>
-      <c r="F6" s="244"/>
-      <c r="G6" s="244"/>
-      <c r="H6" s="244"/>
-      <c r="I6" s="244"/>
-      <c r="J6" s="244"/>
-      <c r="K6" s="245"/>
+      <c r="B6" s="187"/>
+      <c r="C6" s="187"/>
+      <c r="D6" s="187"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="187"/>
+      <c r="G6" s="187"/>
+      <c r="H6" s="187"/>
+      <c r="I6" s="187"/>
+      <c r="J6" s="187"/>
+      <c r="K6" s="188"/>
     </row>
     <row r="7" spans="1:11" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="94" t="s">
+      <c r="A7" s="173" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="95"/>
-      <c r="C7" s="95"/>
-      <c r="D7" s="95"/>
-      <c r="E7" s="246"/>
-      <c r="F7" s="247"/>
-      <c r="G7" s="247"/>
-      <c r="H7" s="247"/>
-      <c r="I7" s="247"/>
-      <c r="J7" s="247"/>
-      <c r="K7" s="248"/>
+      <c r="B7" s="174"/>
+      <c r="C7" s="174"/>
+      <c r="D7" s="174"/>
+      <c r="E7" s="189"/>
+      <c r="F7" s="190"/>
+      <c r="G7" s="190"/>
+      <c r="H7" s="190"/>
+      <c r="I7" s="190"/>
+      <c r="J7" s="190"/>
+      <c r="K7" s="191"/>
     </row>
     <row r="8" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="94" t="s">
+      <c r="A8" s="173" t="s">
         <v>58</v>
       </c>
-      <c r="B8" s="95"/>
-      <c r="C8" s="95"/>
-      <c r="D8" s="95"/>
-      <c r="E8" s="249"/>
-      <c r="F8" s="250"/>
-      <c r="G8" s="250"/>
-      <c r="H8" s="250"/>
-      <c r="I8" s="250"/>
-      <c r="J8" s="250"/>
-      <c r="K8" s="251"/>
+      <c r="B8" s="174"/>
+      <c r="C8" s="174"/>
+      <c r="D8" s="174"/>
+      <c r="E8" s="192"/>
+      <c r="F8" s="193"/>
+      <c r="G8" s="193"/>
+      <c r="H8" s="193"/>
+      <c r="I8" s="193"/>
+      <c r="J8" s="193"/>
+      <c r="K8" s="194"/>
     </row>
     <row r="9" spans="1:11" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="57" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="B9" s="37"/>
       <c r="C9" s="37"/>
@@ -4014,266 +3900,270 @@
       <c r="K11" s="42"/>
     </row>
     <row r="12" spans="1:11" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="205" t="s">
+      <c r="A12" s="198" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="206"/>
-      <c r="C12" s="206"/>
-      <c r="D12" s="206"/>
-      <c r="E12" s="206"/>
-      <c r="F12" s="206"/>
-      <c r="G12" s="206"/>
-      <c r="H12" s="206"/>
-      <c r="I12" s="206"/>
-      <c r="J12" s="206"/>
-      <c r="K12" s="207"/>
+      <c r="B12" s="199"/>
+      <c r="C12" s="199"/>
+      <c r="D12" s="199"/>
+      <c r="E12" s="199"/>
+      <c r="F12" s="199"/>
+      <c r="G12" s="199"/>
+      <c r="H12" s="199"/>
+      <c r="I12" s="199"/>
+      <c r="J12" s="199"/>
+      <c r="K12" s="200"/>
     </row>
     <row r="13" spans="1:11" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="203" t="s">
+      <c r="A13" s="201" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="204"/>
-      <c r="C13" s="204" t="s">
+      <c r="B13" s="202"/>
+      <c r="C13" s="202" t="s">
         <v>61</v>
       </c>
-      <c r="D13" s="204"/>
-      <c r="E13" s="204"/>
-      <c r="F13" s="204"/>
-      <c r="G13" s="204" t="s">
+      <c r="D13" s="202"/>
+      <c r="E13" s="202"/>
+      <c r="F13" s="202"/>
+      <c r="G13" s="202" t="s">
         <v>60</v>
       </c>
-      <c r="H13" s="204"/>
-      <c r="I13" s="204"/>
-      <c r="J13" s="204"/>
-      <c r="K13" s="208"/>
+      <c r="H13" s="202"/>
+      <c r="I13" s="202"/>
+      <c r="J13" s="202"/>
+      <c r="K13" s="246"/>
     </row>
     <row r="14" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="91" t="s">
+      <c r="A14" s="170" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="193"/>
-      <c r="C14" s="199"/>
-      <c r="D14" s="199"/>
-      <c r="E14" s="199"/>
-      <c r="F14" s="199"/>
-      <c r="G14" s="199"/>
-      <c r="H14" s="199"/>
-      <c r="I14" s="199"/>
-      <c r="J14" s="199"/>
-      <c r="K14" s="200"/>
+      <c r="B14" s="233"/>
+      <c r="C14" s="185"/>
+      <c r="D14" s="185"/>
+      <c r="E14" s="185"/>
+      <c r="F14" s="185"/>
+      <c r="G14" s="185"/>
+      <c r="H14" s="185"/>
+      <c r="I14" s="185"/>
+      <c r="J14" s="185"/>
+      <c r="K14" s="244"/>
     </row>
     <row r="15" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="91" t="s">
+      <c r="A15" s="170" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="193"/>
-      <c r="C15" s="199"/>
-      <c r="D15" s="199"/>
-      <c r="E15" s="199"/>
-      <c r="F15" s="199"/>
-      <c r="G15" s="199"/>
-      <c r="H15" s="199"/>
-      <c r="I15" s="199"/>
-      <c r="J15" s="199"/>
-      <c r="K15" s="200"/>
+      <c r="B15" s="233"/>
+      <c r="C15" s="185"/>
+      <c r="D15" s="185"/>
+      <c r="E15" s="185"/>
+      <c r="F15" s="185"/>
+      <c r="G15" s="185"/>
+      <c r="H15" s="185"/>
+      <c r="I15" s="185"/>
+      <c r="J15" s="185"/>
+      <c r="K15" s="244"/>
     </row>
     <row r="16" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="194" t="s">
+      <c r="A16" s="239" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="195"/>
-      <c r="C16" s="198"/>
-      <c r="D16" s="198"/>
-      <c r="E16" s="198"/>
-      <c r="F16" s="198"/>
-      <c r="G16" s="198"/>
-      <c r="H16" s="198"/>
-      <c r="I16" s="198"/>
-      <c r="J16" s="198"/>
-      <c r="K16" s="201"/>
+      <c r="B16" s="240"/>
+      <c r="C16" s="243"/>
+      <c r="D16" s="243"/>
+      <c r="E16" s="243"/>
+      <c r="F16" s="243"/>
+      <c r="G16" s="243"/>
+      <c r="H16" s="243"/>
+      <c r="I16" s="243"/>
+      <c r="J16" s="243"/>
+      <c r="K16" s="245"/>
     </row>
     <row r="17" spans="1:11" s="7" customFormat="1" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="43"/>
       <c r="K17" s="44"/>
     </row>
     <row r="18" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="205" t="s">
+      <c r="A18" s="198" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="206"/>
-      <c r="C18" s="206"/>
-      <c r="D18" s="206"/>
-      <c r="E18" s="206"/>
-      <c r="F18" s="206"/>
-      <c r="G18" s="206"/>
-      <c r="H18" s="206"/>
-      <c r="I18" s="206"/>
-      <c r="J18" s="206"/>
-      <c r="K18" s="207"/>
+      <c r="B18" s="199"/>
+      <c r="C18" s="199"/>
+      <c r="D18" s="199"/>
+      <c r="E18" s="199"/>
+      <c r="F18" s="199"/>
+      <c r="G18" s="199"/>
+      <c r="H18" s="199"/>
+      <c r="I18" s="199"/>
+      <c r="J18" s="199"/>
+      <c r="K18" s="200"/>
     </row>
     <row r="19" spans="1:11" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="203" t="s">
+      <c r="A19" s="201" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="204"/>
-      <c r="C19" s="196" t="s">
+      <c r="B19" s="202"/>
+      <c r="C19" s="241" t="s">
         <v>65</v>
       </c>
-      <c r="D19" s="196"/>
-      <c r="E19" s="196"/>
-      <c r="F19" s="196"/>
-      <c r="G19" s="196"/>
-      <c r="H19" s="196"/>
-      <c r="I19" s="196"/>
-      <c r="J19" s="196"/>
-      <c r="K19" s="197"/>
+      <c r="D19" s="241"/>
+      <c r="E19" s="241"/>
+      <c r="F19" s="241"/>
+      <c r="G19" s="241"/>
+      <c r="H19" s="241"/>
+      <c r="I19" s="241"/>
+      <c r="J19" s="241"/>
+      <c r="K19" s="242"/>
     </row>
     <row r="20" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="94" t="s">
+      <c r="A20" s="173" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="95"/>
-      <c r="C20" s="202"/>
-      <c r="D20" s="202"/>
-      <c r="E20" s="202"/>
-      <c r="F20" s="202"/>
-      <c r="G20" s="202"/>
-      <c r="H20" s="202"/>
-      <c r="I20" s="202"/>
-      <c r="J20" s="202"/>
-      <c r="K20" s="253" t="s">
+      <c r="B20" s="174"/>
+      <c r="C20" s="235" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" s="235"/>
+      <c r="E20" s="235"/>
+      <c r="F20" s="235"/>
+      <c r="G20" s="235"/>
+      <c r="H20" s="235"/>
+      <c r="I20" s="235"/>
+      <c r="J20" s="235"/>
+      <c r="K20" s="203" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="94" t="s">
+      <c r="A21" s="173" t="s">
         <v>63</v>
       </c>
-      <c r="B21" s="95"/>
-      <c r="C21" s="202"/>
-      <c r="D21" s="202"/>
-      <c r="E21" s="202"/>
-      <c r="F21" s="202"/>
-      <c r="G21" s="202"/>
-      <c r="H21" s="202"/>
-      <c r="I21" s="202"/>
-      <c r="J21" s="202"/>
-      <c r="K21" s="254"/>
+      <c r="B21" s="174"/>
+      <c r="C21" s="235" t="s">
+        <v>115</v>
+      </c>
+      <c r="D21" s="235"/>
+      <c r="E21" s="235"/>
+      <c r="F21" s="235"/>
+      <c r="G21" s="235"/>
+      <c r="H21" s="235"/>
+      <c r="I21" s="235"/>
+      <c r="J21" s="235"/>
+      <c r="K21" s="204"/>
     </row>
     <row r="22" spans="1:11" s="7" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="210"/>
-      <c r="B22" s="211"/>
-      <c r="C22" s="202"/>
-      <c r="D22" s="202"/>
-      <c r="E22" s="202"/>
-      <c r="F22" s="202"/>
-      <c r="G22" s="202"/>
-      <c r="H22" s="202"/>
-      <c r="I22" s="202"/>
-      <c r="J22" s="202"/>
-      <c r="K22" s="255"/>
+      <c r="A22" s="234"/>
+      <c r="B22" s="184"/>
+      <c r="C22" s="235"/>
+      <c r="D22" s="235"/>
+      <c r="E22" s="235"/>
+      <c r="F22" s="235"/>
+      <c r="G22" s="235"/>
+      <c r="H22" s="235"/>
+      <c r="I22" s="235"/>
+      <c r="J22" s="235"/>
+      <c r="K22" s="205"/>
     </row>
     <row r="23" spans="1:11" s="1" customFormat="1" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="45"/>
       <c r="K23" s="46"/>
     </row>
     <row r="24" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="128" t="s">
+      <c r="A24" s="117" t="s">
         <v>66</v>
       </c>
-      <c r="B24" s="209"/>
-      <c r="C24" s="209"/>
-      <c r="D24" s="129"/>
-      <c r="E24" s="212" t="s">
+      <c r="B24" s="196"/>
+      <c r="C24" s="196"/>
+      <c r="D24" s="118"/>
+      <c r="E24" s="195" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="209"/>
-      <c r="G24" s="129"/>
-      <c r="H24" s="212" t="s">
+      <c r="F24" s="196"/>
+      <c r="G24" s="118"/>
+      <c r="H24" s="195" t="s">
         <v>40</v>
       </c>
-      <c r="I24" s="209"/>
-      <c r="J24" s="209"/>
-      <c r="K24" s="252"/>
+      <c r="I24" s="196"/>
+      <c r="J24" s="196"/>
+      <c r="K24" s="197"/>
     </row>
     <row r="25" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="227" t="s">
+      <c r="A25" s="208" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="228"/>
-      <c r="C25" s="218" t="s">
+      <c r="B25" s="209"/>
+      <c r="C25" s="179" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="218"/>
-      <c r="E25" s="186"/>
-      <c r="F25" s="186"/>
-      <c r="G25" s="186"/>
-      <c r="H25" s="213"/>
-      <c r="I25" s="214"/>
-      <c r="J25" s="214"/>
-      <c r="K25" s="215"/>
+      <c r="D25" s="179"/>
+      <c r="E25" s="79"/>
+      <c r="F25" s="79"/>
+      <c r="G25" s="79"/>
+      <c r="H25" s="214"/>
+      <c r="I25" s="215"/>
+      <c r="J25" s="215"/>
+      <c r="K25" s="224"/>
     </row>
     <row r="26" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="229"/>
-      <c r="B26" s="230"/>
-      <c r="C26" s="218" t="s">
+      <c r="A26" s="210"/>
+      <c r="B26" s="211"/>
+      <c r="C26" s="179" t="s">
         <v>50</v>
       </c>
-      <c r="D26" s="218"/>
-      <c r="E26" s="213"/>
-      <c r="F26" s="214"/>
-      <c r="G26" s="233"/>
-      <c r="H26" s="213"/>
-      <c r="I26" s="214"/>
-      <c r="J26" s="214"/>
-      <c r="K26" s="215"/>
+      <c r="D26" s="179"/>
+      <c r="E26" s="214"/>
+      <c r="F26" s="215"/>
+      <c r="G26" s="216"/>
+      <c r="H26" s="214"/>
+      <c r="I26" s="215"/>
+      <c r="J26" s="215"/>
+      <c r="K26" s="224"/>
     </row>
     <row r="27" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="231"/>
-      <c r="B27" s="232"/>
-      <c r="C27" s="218" t="s">
+      <c r="A27" s="212"/>
+      <c r="B27" s="213"/>
+      <c r="C27" s="179" t="s">
         <v>42</v>
       </c>
-      <c r="D27" s="218"/>
-      <c r="E27" s="125"/>
-      <c r="F27" s="125"/>
-      <c r="G27" s="125"/>
-      <c r="H27" s="138"/>
-      <c r="I27" s="138"/>
-      <c r="J27" s="138"/>
-      <c r="K27" s="216"/>
+      <c r="D27" s="179"/>
+      <c r="E27" s="70"/>
+      <c r="F27" s="70"/>
+      <c r="G27" s="70"/>
+      <c r="H27" s="78"/>
+      <c r="I27" s="78"/>
+      <c r="J27" s="78"/>
+      <c r="K27" s="225"/>
     </row>
     <row r="28" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="239" t="s">
+      <c r="A28" s="180" t="s">
         <v>43</v>
       </c>
-      <c r="B28" s="240"/>
-      <c r="C28" s="95" t="s">
+      <c r="B28" s="181"/>
+      <c r="C28" s="174" t="s">
         <v>41</v>
       </c>
-      <c r="D28" s="95"/>
-      <c r="E28" s="186"/>
-      <c r="F28" s="186"/>
-      <c r="G28" s="186"/>
-      <c r="H28" s="213"/>
-      <c r="I28" s="214"/>
-      <c r="J28" s="214"/>
-      <c r="K28" s="215"/>
+      <c r="D28" s="174"/>
+      <c r="E28" s="79"/>
+      <c r="F28" s="79"/>
+      <c r="G28" s="79"/>
+      <c r="H28" s="214"/>
+      <c r="I28" s="215"/>
+      <c r="J28" s="215"/>
+      <c r="K28" s="224"/>
     </row>
     <row r="29" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="241"/>
-      <c r="B29" s="242"/>
-      <c r="C29" s="211" t="s">
+      <c r="A29" s="182"/>
+      <c r="B29" s="183"/>
+      <c r="C29" s="184" t="s">
         <v>42</v>
       </c>
-      <c r="D29" s="211"/>
-      <c r="E29" s="225"/>
-      <c r="F29" s="225"/>
-      <c r="G29" s="225"/>
-      <c r="H29" s="140"/>
-      <c r="I29" s="140"/>
-      <c r="J29" s="140"/>
-      <c r="K29" s="217"/>
+      <c r="D29" s="184"/>
+      <c r="E29" s="206"/>
+      <c r="F29" s="206"/>
+      <c r="G29" s="206"/>
+      <c r="H29" s="73"/>
+      <c r="I29" s="73"/>
+      <c r="J29" s="73"/>
+      <c r="K29" s="226"/>
     </row>
     <row r="30" spans="1:11" s="1" customFormat="1" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="47"/>
@@ -4289,229 +4179,229 @@
       <c r="K30" s="48"/>
     </row>
     <row r="31" spans="1:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="85" t="s">
+      <c r="A31" s="164" t="s">
         <v>51</v>
       </c>
-      <c r="B31" s="86"/>
-      <c r="C31" s="86"/>
-      <c r="D31" s="86"/>
-      <c r="E31" s="86"/>
-      <c r="F31" s="86"/>
-      <c r="G31" s="86"/>
-      <c r="H31" s="86"/>
-      <c r="I31" s="86"/>
-      <c r="J31" s="86"/>
-      <c r="K31" s="87"/>
+      <c r="B31" s="165"/>
+      <c r="C31" s="165"/>
+      <c r="D31" s="165"/>
+      <c r="E31" s="165"/>
+      <c r="F31" s="165"/>
+      <c r="G31" s="165"/>
+      <c r="H31" s="165"/>
+      <c r="I31" s="165"/>
+      <c r="J31" s="165"/>
+      <c r="K31" s="166"/>
     </row>
     <row r="32" spans="1:11" s="14" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="226" t="s">
+      <c r="A32" s="207" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="96"/>
-      <c r="C32" s="96"/>
-      <c r="D32" s="96"/>
-      <c r="E32" s="96"/>
-      <c r="F32" s="96"/>
-      <c r="G32" s="96"/>
-      <c r="H32" s="96"/>
-      <c r="I32" s="96"/>
-      <c r="J32" s="96"/>
-      <c r="K32" s="97"/>
+      <c r="B32" s="175"/>
+      <c r="C32" s="175"/>
+      <c r="D32" s="175"/>
+      <c r="E32" s="175"/>
+      <c r="F32" s="175"/>
+      <c r="G32" s="175"/>
+      <c r="H32" s="175"/>
+      <c r="I32" s="175"/>
+      <c r="J32" s="175"/>
+      <c r="K32" s="176"/>
     </row>
     <row r="33" spans="1:11" s="14" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="94" t="s">
+      <c r="A33" s="173" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="95"/>
-      <c r="C33" s="95"/>
-      <c r="D33" s="95"/>
-      <c r="E33" s="95"/>
-      <c r="F33" s="95"/>
-      <c r="G33" s="95"/>
-      <c r="H33" s="95"/>
-      <c r="I33" s="95"/>
-      <c r="J33" s="95"/>
-      <c r="K33" s="98"/>
+      <c r="B33" s="174"/>
+      <c r="C33" s="174"/>
+      <c r="D33" s="174"/>
+      <c r="E33" s="174"/>
+      <c r="F33" s="174"/>
+      <c r="G33" s="174"/>
+      <c r="H33" s="174"/>
+      <c r="I33" s="174"/>
+      <c r="J33" s="174"/>
+      <c r="K33" s="177"/>
     </row>
     <row r="34" spans="1:11" s="1" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="234" t="s">
+      <c r="A34" s="217" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="235"/>
-      <c r="C34" s="236"/>
-      <c r="D34" s="234" t="s">
+      <c r="B34" s="218"/>
+      <c r="C34" s="219"/>
+      <c r="D34" s="217" t="s">
         <v>86</v>
       </c>
-      <c r="E34" s="235"/>
-      <c r="F34" s="235"/>
-      <c r="G34" s="236"/>
-      <c r="H34" s="234" t="s">
-        <v>90</v>
-      </c>
-      <c r="I34" s="235"/>
-      <c r="J34" s="235"/>
-      <c r="K34" s="237"/>
+      <c r="E34" s="218"/>
+      <c r="F34" s="218"/>
+      <c r="G34" s="219"/>
+      <c r="H34" s="217" t="s">
+        <v>114</v>
+      </c>
+      <c r="I34" s="218"/>
+      <c r="J34" s="218"/>
+      <c r="K34" s="220"/>
     </row>
     <row r="35" spans="1:11" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="94" t="s">
+      <c r="A35" s="173" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="95"/>
-      <c r="C35" s="95"/>
-      <c r="D35" s="222"/>
-      <c r="E35" s="223"/>
-      <c r="F35" s="223"/>
-      <c r="G35" s="223"/>
-      <c r="H35" s="223"/>
-      <c r="I35" s="223"/>
-      <c r="J35" s="223"/>
-      <c r="K35" s="224"/>
+      <c r="B35" s="174"/>
+      <c r="C35" s="174"/>
+      <c r="D35" s="230"/>
+      <c r="E35" s="231"/>
+      <c r="F35" s="231"/>
+      <c r="G35" s="231"/>
+      <c r="H35" s="231"/>
+      <c r="I35" s="231"/>
+      <c r="J35" s="231"/>
+      <c r="K35" s="232"/>
     </row>
     <row r="36" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="94" t="s">
+      <c r="A36" s="173" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="95"/>
-      <c r="C36" s="95"/>
-      <c r="D36" s="95"/>
-      <c r="E36" s="95"/>
-      <c r="F36" s="95"/>
-      <c r="G36" s="95"/>
-      <c r="H36" s="95"/>
-      <c r="I36" s="95"/>
-      <c r="J36" s="95"/>
-      <c r="K36" s="98"/>
+      <c r="B36" s="174"/>
+      <c r="C36" s="174"/>
+      <c r="D36" s="174"/>
+      <c r="E36" s="174"/>
+      <c r="F36" s="174"/>
+      <c r="G36" s="174"/>
+      <c r="H36" s="174"/>
+      <c r="I36" s="174"/>
+      <c r="J36" s="174"/>
+      <c r="K36" s="177"/>
     </row>
     <row r="37" spans="1:11" s="19" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="94" t="s">
+      <c r="A37" s="173" t="s">
         <v>47</v>
       </c>
-      <c r="B37" s="95"/>
-      <c r="C37" s="95"/>
-      <c r="D37" s="95"/>
-      <c r="E37" s="95"/>
-      <c r="F37" s="95"/>
-      <c r="G37" s="95"/>
-      <c r="H37" s="95"/>
-      <c r="I37" s="95"/>
-      <c r="J37" s="95"/>
-      <c r="K37" s="98"/>
+      <c r="B37" s="174"/>
+      <c r="C37" s="174"/>
+      <c r="D37" s="174"/>
+      <c r="E37" s="174"/>
+      <c r="F37" s="174"/>
+      <c r="G37" s="174"/>
+      <c r="H37" s="174"/>
+      <c r="I37" s="174"/>
+      <c r="J37" s="174"/>
+      <c r="K37" s="177"/>
     </row>
     <row r="38" spans="1:11" s="19" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="94" t="s">
+      <c r="A38" s="173" t="s">
         <v>16</v>
       </c>
-      <c r="B38" s="95"/>
-      <c r="C38" s="95"/>
-      <c r="D38" s="95"/>
-      <c r="E38" s="95"/>
-      <c r="F38" s="95"/>
-      <c r="G38" s="95"/>
-      <c r="H38" s="95"/>
-      <c r="I38" s="95"/>
-      <c r="J38" s="95"/>
-      <c r="K38" s="98"/>
+      <c r="B38" s="174"/>
+      <c r="C38" s="174"/>
+      <c r="D38" s="174"/>
+      <c r="E38" s="174"/>
+      <c r="F38" s="174"/>
+      <c r="G38" s="174"/>
+      <c r="H38" s="174"/>
+      <c r="I38" s="174"/>
+      <c r="J38" s="174"/>
+      <c r="K38" s="177"/>
     </row>
     <row r="39" spans="1:11" s="19" customFormat="1" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="94" t="s">
+      <c r="A39" s="173" t="s">
         <v>17</v>
       </c>
-      <c r="B39" s="95"/>
-      <c r="C39" s="95"/>
-      <c r="D39" s="95"/>
-      <c r="E39" s="95"/>
-      <c r="F39" s="95"/>
-      <c r="G39" s="95"/>
-      <c r="H39" s="95"/>
-      <c r="I39" s="95"/>
-      <c r="J39" s="95"/>
-      <c r="K39" s="98"/>
+      <c r="B39" s="174"/>
+      <c r="C39" s="174"/>
+      <c r="D39" s="174"/>
+      <c r="E39" s="174"/>
+      <c r="F39" s="174"/>
+      <c r="G39" s="174"/>
+      <c r="H39" s="174"/>
+      <c r="I39" s="174"/>
+      <c r="J39" s="174"/>
+      <c r="K39" s="177"/>
     </row>
     <row r="40" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="219" t="s">
+      <c r="A40" s="227" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="220"/>
-      <c r="C40" s="220"/>
-      <c r="D40" s="220"/>
-      <c r="E40" s="220"/>
-      <c r="F40" s="220"/>
-      <c r="G40" s="220"/>
-      <c r="H40" s="220"/>
-      <c r="I40" s="220"/>
-      <c r="J40" s="220"/>
-      <c r="K40" s="221"/>
+      <c r="B40" s="228"/>
+      <c r="C40" s="228"/>
+      <c r="D40" s="228"/>
+      <c r="E40" s="228"/>
+      <c r="F40" s="228"/>
+      <c r="G40" s="228"/>
+      <c r="H40" s="228"/>
+      <c r="I40" s="228"/>
+      <c r="J40" s="228"/>
+      <c r="K40" s="229"/>
     </row>
     <row r="41" spans="1:11" s="1" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="187" t="s">
-        <v>98</v>
-      </c>
-      <c r="B41" s="188"/>
-      <c r="C41" s="188"/>
-      <c r="D41" s="188"/>
-      <c r="E41" s="188"/>
-      <c r="F41" s="188"/>
-      <c r="G41" s="188"/>
-      <c r="H41" s="188"/>
-      <c r="I41" s="188"/>
-      <c r="J41" s="188"/>
-      <c r="K41" s="189"/>
+      <c r="A41" s="221" t="s">
+        <v>97</v>
+      </c>
+      <c r="B41" s="222"/>
+      <c r="C41" s="222"/>
+      <c r="D41" s="222"/>
+      <c r="E41" s="222"/>
+      <c r="F41" s="222"/>
+      <c r="G41" s="222"/>
+      <c r="H41" s="222"/>
+      <c r="I41" s="222"/>
+      <c r="J41" s="222"/>
+      <c r="K41" s="223"/>
     </row>
     <row r="42" spans="1:11" s="1" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="187" t="s">
-        <v>115</v>
-      </c>
-      <c r="B42" s="188"/>
-      <c r="C42" s="188"/>
-      <c r="D42" s="188"/>
-      <c r="E42" s="188"/>
-      <c r="F42" s="188"/>
-      <c r="G42" s="188"/>
-      <c r="H42" s="188"/>
-      <c r="I42" s="188"/>
-      <c r="J42" s="188"/>
-      <c r="K42" s="189"/>
+      <c r="A42" s="221" t="s">
+        <v>113</v>
+      </c>
+      <c r="B42" s="222"/>
+      <c r="C42" s="222"/>
+      <c r="D42" s="222"/>
+      <c r="E42" s="222"/>
+      <c r="F42" s="222"/>
+      <c r="G42" s="222"/>
+      <c r="H42" s="222"/>
+      <c r="I42" s="222"/>
+      <c r="J42" s="222"/>
+      <c r="K42" s="223"/>
     </row>
     <row r="43" spans="1:11" s="1" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="187" t="s">
+      <c r="A43" s="221" t="s">
         <v>87</v>
       </c>
-      <c r="B43" s="188"/>
-      <c r="C43" s="188"/>
-      <c r="D43" s="188"/>
-      <c r="E43" s="188"/>
-      <c r="F43" s="188"/>
-      <c r="G43" s="188"/>
-      <c r="H43" s="188"/>
-      <c r="I43" s="188"/>
-      <c r="J43" s="188"/>
-      <c r="K43" s="189"/>
+      <c r="B43" s="222"/>
+      <c r="C43" s="222"/>
+      <c r="D43" s="222"/>
+      <c r="E43" s="222"/>
+      <c r="F43" s="222"/>
+      <c r="G43" s="222"/>
+      <c r="H43" s="222"/>
+      <c r="I43" s="222"/>
+      <c r="J43" s="222"/>
+      <c r="K43" s="223"/>
     </row>
     <row r="44" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="187"/>
-      <c r="B44" s="188"/>
-      <c r="C44" s="188"/>
-      <c r="D44" s="188"/>
-      <c r="E44" s="188"/>
-      <c r="F44" s="188"/>
-      <c r="G44" s="188"/>
-      <c r="H44" s="188"/>
-      <c r="I44" s="188"/>
-      <c r="J44" s="188"/>
-      <c r="K44" s="189"/>
+      <c r="A44" s="221"/>
+      <c r="B44" s="222"/>
+      <c r="C44" s="222"/>
+      <c r="D44" s="222"/>
+      <c r="E44" s="222"/>
+      <c r="F44" s="222"/>
+      <c r="G44" s="222"/>
+      <c r="H44" s="222"/>
+      <c r="I44" s="222"/>
+      <c r="J44" s="222"/>
+      <c r="K44" s="223"/>
     </row>
     <row r="45" spans="1:11" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="190"/>
-      <c r="B45" s="191"/>
-      <c r="C45" s="191"/>
-      <c r="D45" s="191"/>
-      <c r="E45" s="191"/>
-      <c r="F45" s="191"/>
-      <c r="G45" s="191"/>
-      <c r="H45" s="191"/>
-      <c r="I45" s="191"/>
-      <c r="J45" s="191"/>
-      <c r="K45" s="192"/>
+      <c r="A45" s="236"/>
+      <c r="B45" s="237"/>
+      <c r="C45" s="237"/>
+      <c r="D45" s="237"/>
+      <c r="E45" s="237"/>
+      <c r="F45" s="237"/>
+      <c r="G45" s="237"/>
+      <c r="H45" s="237"/>
+      <c r="I45" s="237"/>
+      <c r="J45" s="237"/>
+      <c r="K45" s="238"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
@@ -4530,6 +4420,58 @@
     </row>
   </sheetData>
   <mergeCells count="68">
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A45:K45"/>
+    <mergeCell ref="D2:K3"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C19:K19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="G14:K14"/>
+    <mergeCell ref="G15:K15"/>
+    <mergeCell ref="G16:K16"/>
+    <mergeCell ref="C20:J20"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A18:K18"/>
+    <mergeCell ref="G13:K13"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C21:J21"/>
+    <mergeCell ref="C22:J22"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="H27:K27"/>
+    <mergeCell ref="H28:K28"/>
+    <mergeCell ref="H29:K29"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A40:K40"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="D35:K35"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A38:K38"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="H26:K26"/>
+    <mergeCell ref="A39:K39"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A33:K33"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="A32:K32"/>
+    <mergeCell ref="A25:B27"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D34:G34"/>
+    <mergeCell ref="H34:K34"/>
     <mergeCell ref="D4:J4"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="A31:K31"/>
@@ -4546,58 +4488,6 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="K20:K22"/>
     <mergeCell ref="C15:F15"/>
-    <mergeCell ref="A36:K36"/>
-    <mergeCell ref="A33:K33"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="A32:K32"/>
-    <mergeCell ref="A25:B27"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:G34"/>
-    <mergeCell ref="H34:K34"/>
-    <mergeCell ref="A43:K43"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="H27:K27"/>
-    <mergeCell ref="H28:K28"/>
-    <mergeCell ref="H29:K29"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A40:K40"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="D35:K35"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A38:K38"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="A37:K37"/>
-    <mergeCell ref="H26:K26"/>
-    <mergeCell ref="A39:K39"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C21:J21"/>
-    <mergeCell ref="C22:J22"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A45:K45"/>
-    <mergeCell ref="D2:K3"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C19:K19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="G14:K14"/>
-    <mergeCell ref="G15:K15"/>
-    <mergeCell ref="G16:K16"/>
-    <mergeCell ref="C20:J20"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A18:K18"/>
-    <mergeCell ref="G13:K13"/>
-    <mergeCell ref="C13:F13"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>